<commit_message>
fix: update address and telecom use mapping in Patient and Organization resources of HL7 files #2841
</commit_message>
<xml_diff>
--- a/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
+++ b/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" tabRatio="753" firstSheet="1" activeTab="5"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="753" firstSheet="1" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="669" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="439">
   <si>
     <t>FHIR Resources</t>
   </si>
@@ -853,17 +853,17 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF00B050"/>
         <rFont val="Calibri"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-H, HP, HV -&gt; home
-WP, O -&gt; work
-TMP, C -&gt; temp
-BAD -&gt; old
-All Others (DIR, PUB, AS, EC, MC, PG) -&gt; home</t>
+F, H, M, P, BDL -&gt; home
+B, O, S, SH, RH, TM -&gt; work
+V, C -&gt; temp
+BA -&gt; old
+All Others -&gt; home</t>
     </r>
   </si>
   <si>
@@ -889,27 +889,8 @@
     <t>telecom -&gt; use</t>
   </si>
   <si>
-    <t>PID.13.2, PID.14.2, PID.40.2</t>
-  </si>
-  <si>
-    <r>
-      <t>telecom -&gt; use Mapping</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-AS, DIR, PUB, WP -&gt; work
-H, HP, HV, EC -&gt; home
-MC, PG -&gt; mobile
-TMP -&gt; temp
-BAD -&gt; old</t>
-    </r>
+    <t>PID.13 -&gt; 'home'
+PID.14 and PID.40 -&gt; 'work'</t>
   </si>
   <si>
     <t>extension -&gt; extension -&gt; url</t>
@@ -3862,27 +3843,7 @@
     </r>
   </si>
   <si>
-    <t>ORC.23.2</t>
-  </si>
-  <si>
-    <r>
-      <t>telecom -&gt; use Mapping</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-AS, DIR, PUB, WP -&gt; work
-MC, PG -&gt; mobile
-TMP -&gt; temp
-BAD -&gt; old
-All others (H, HP, HV, EC) -&gt; work</t>
-    </r>
+    <t>"work"</t>
   </si>
   <si>
     <t>ORC.22.1 + OR.C22.2 + ORC.22.3 + ORC.22.4 + ORC.22.5 + ORC.22.6</t>
@@ -3908,17 +3869,17 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF00B050"/>
         <rFont val="Calibri"/>
         <charset val="134"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-WP -&gt; work
-BA -&gt; billing
-TMP -&gt; temp
-BAD -&gt; old
-All Others (H, HP, HV, DIR, PUB, AS, EC, MC, PG) -&gt; work</t>
+F, H, M, P, BDL -&gt; home
+B, O, S, SH, RH, TM -&gt; work
+V, C -&gt; temp
+BA -&gt; old
+All Others -&gt; work</t>
     </r>
   </si>
   <si>
@@ -5084,7 +5045,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="58">
+  <fonts count="59">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -5235,6 +5196,15 @@
       <u/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5448,20 +5418,13 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
-      <u/>
-      <sz val="10"/>
+      <b/>
+      <sz val="11"/>
       <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -5470,6 +5433,21 @@
       <b/>
       <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -5488,19 +5466,11 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <u/>
+      <sz val="10"/>
       <color rgb="FF00B050"/>
       <name val="Calibri"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="40">
@@ -5865,151 +5835,148 @@
     <xf numFmtId="179" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="45" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="46" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -6018,17 +5985,20 @@
     <xf numFmtId="0" fontId="48" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="49" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6167,6 +6137,9 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -6176,7 +6149,10 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -6200,7 +6176,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -6303,7 +6279,7 @@
     <cellStyle name="Warning" xfId="59"/>
   </cellStyles>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{5E6FBFC4-12AA-4B25-8E12-E7CF585DDB12}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{E3B77C8E-14A8-4A8F-831C-BD0090FCDAAF}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -6572,68 +6548,68 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11.8545454545455" defaultRowHeight="14.5" outlineLevelRow="7" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="11.8571428571429" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="14.2818181818182" style="66" customWidth="1"/>
+    <col min="1" max="1" width="14.2857142857143" style="68" customWidth="1"/>
     <col min="2" max="2" width="47" customWidth="1"/>
-    <col min="3" max="3" width="123.572727272727" customWidth="1"/>
+    <col min="3" max="3" width="123.571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="62"/>
-      <c r="C1" s="62"/>
+      <c r="B1" s="64"/>
+      <c r="C1" s="64"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="62"/>
-      <c r="B2" s="62" t="s">
+      <c r="A2" s="64"/>
+      <c r="B2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="55" t="s">
+      <c r="C2" s="57" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="62"/>
-      <c r="B3" s="62" t="s">
+      <c r="A3" s="64"/>
+      <c r="B3" s="64" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="57" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="62"/>
-      <c r="B4" s="62" t="s">
+      <c r="A4" s="64"/>
+      <c r="B4" s="64" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="57" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" ht="43.5" spans="1:3">
-      <c r="A5" s="62"/>
-      <c r="B5" s="62" t="s">
+    <row r="5" ht="45" spans="1:3">
+      <c r="A5" s="64"/>
+      <c r="B5" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="65" t="s">
+      <c r="C5" s="67" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="62"/>
-      <c r="B6" s="65" t="s">
+      <c r="A6" s="64"/>
+      <c r="B6" s="67" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="55" t="s">
+      <c r="C6" s="57" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="62"/>
-      <c r="B7" s="62" t="s">
+      <c r="A7" s="64"/>
+      <c r="B7" s="64" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="12" t="s">
@@ -6641,8 +6617,8 @@
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" s="62"/>
-      <c r="B8" s="62"/>
+      <c r="A8" s="64"/>
+      <c r="B8" s="64"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1.39370078740157" bottom="1.39370078740157" header="1" footer="1"/>
@@ -6655,15 +6631,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" style="2" customWidth="1"/>
-    <col min="2" max="2" width="33.5727272727273" style="2" customWidth="1"/>
-    <col min="3" max="3" width="49.6636363636364" style="2" customWidth="1"/>
-    <col min="4" max="4" width="56.5545454545455" style="2" customWidth="1"/>
-    <col min="5" max="5" width="53.2818181818182" style="2" customWidth="1"/>
-    <col min="6" max="6" width="47.5727272727273" style="2" customWidth="1"/>
-    <col min="7" max="16384" width="9.14545454545454" style="2"/>
+    <col min="1" max="1" width="14.7142857142857" style="2" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" style="2" customWidth="1"/>
+    <col min="3" max="3" width="49.6666666666667" style="2" customWidth="1"/>
+    <col min="4" max="4" width="56.552380952381" style="2" customWidth="1"/>
+    <col min="5" max="5" width="53.2857142857143" style="2" customWidth="1"/>
+    <col min="6" max="6" width="47.5714285714286" style="2" customWidth="1"/>
+    <col min="7" max="16384" width="9.14285714285714" style="2"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:6">
@@ -6674,16 +6650,16 @@
         <v>14</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="2" s="2" customFormat="1" ht="17" customHeight="1" spans="1:6">
@@ -6702,7 +6678,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:4">
@@ -6714,7 +6690,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" spans="1:6">
@@ -6729,12 +6705,12 @@
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" s="2" customFormat="1" ht="29" spans="2:6">
+    <row r="6" s="2" customFormat="1" ht="30" spans="2:6">
       <c r="B6" s="7" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -6749,168 +6725,168 @@
         <v>53</v>
       </c>
       <c r="E7" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="8" s="2" customFormat="1" ht="74.25" spans="2:5">
+      <c r="B8" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>421</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="D8" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="E8" s="10" t="s">
         <v>422</v>
-      </c>
-    </row>
-    <row r="8" s="2" customFormat="1" ht="71.5" spans="2:5">
-      <c r="B8" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>423</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="409" customHeight="1" spans="2:5">
       <c r="B9" s="6" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="5" t="s">
+        <v>423</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" s="2" customFormat="1" ht="150" spans="2:5">
+      <c r="B10" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>425</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>426</v>
       </c>
-    </row>
-    <row r="10" s="2" customFormat="1" ht="145" spans="2:5">
-      <c r="B10" s="6" t="s">
-        <v>353</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="8" t="s">
         <v>427</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>428</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="11" s="2" customFormat="1" ht="159.5" spans="2:5">
+    </row>
+    <row r="11" s="2" customFormat="1" ht="180" spans="2:5">
       <c r="B11" s="6" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="2"/>
       <c r="E11" s="11" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="12" s="2" customFormat="1" ht="145" spans="2:5">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="12" s="2" customFormat="1" ht="150" spans="2:5">
       <c r="B12" s="6" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="2"/>
       <c r="E12" s="11" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="13" s="2" customFormat="1" ht="75" spans="2:4">
+      <c r="B13" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="14" s="2" customFormat="1" ht="30" spans="2:3">
+      <c r="B14" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="15" s="2" customFormat="1" ht="45" spans="2:4">
+      <c r="B15" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="13" s="2" customFormat="1" ht="58" spans="2:4">
-      <c r="B13" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>367</v>
-      </c>
-      <c r="D13" s="5" t="s">
+    <row r="16" s="2" customFormat="1" ht="30" spans="2:5">
+      <c r="B16" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="17" s="2" customFormat="1" ht="45" spans="2:4">
+      <c r="B17" s="6" t="s">
         <v>432</v>
       </c>
-    </row>
-    <row r="14" s="2" customFormat="1" ht="29" spans="2:3">
-      <c r="B14" s="6" t="s">
-        <v>254</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="15" s="2" customFormat="1" ht="43.5" spans="2:4">
-      <c r="B15" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="C17" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>433</v>
-      </c>
-    </row>
-    <row r="16" s="2" customFormat="1" ht="29" spans="2:5">
-      <c r="B16" s="6" t="s">
-        <v>372</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>396</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>374</v>
-      </c>
-      <c r="E16" s="14" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="17" s="2" customFormat="1" ht="43.5" spans="2:4">
-      <c r="B17" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>435</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" spans="2:6">
       <c r="B18" s="2" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="E18" s="8"/>
       <c r="F18" s="15" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="19" s="2" customFormat="1" ht="165" spans="2:5">
+      <c r="B19" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="D19" s="5" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="19" s="2" customFormat="1" ht="159.5" spans="2:5">
-      <c r="B19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>438</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>439</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" spans="2:4">
       <c r="B20" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="C20" s="5" t="s">
-        <v>176</v>
-      </c>
       <c r="D20" s="16" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="46" customHeight="1" spans="2:4">
       <c r="B21" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D21" s="16"/>
     </row>
@@ -6928,26 +6904,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7181818181818" style="62" customWidth="1"/>
-    <col min="2" max="2" width="28.2818181818182" style="62" customWidth="1"/>
-    <col min="3" max="3" width="62.7272727272727" style="62" customWidth="1"/>
-    <col min="4" max="4" width="54.5454545454545" style="62" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" style="64" customWidth="1"/>
+    <col min="2" max="2" width="28.2857142857143" style="64" customWidth="1"/>
+    <col min="3" max="3" width="62.7238095238095" style="64" customWidth="1"/>
+    <col min="4" max="4" width="54.5428571428571" style="64" customWidth="1"/>
     <col min="5" max="5" width="57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="63" t="s">
+      <c r="B1" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="63" t="s">
+      <c r="C1" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="63" t="s">
+      <c r="D1" s="65" t="s">
         <v>16</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -6955,82 +6931,82 @@
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="64" t="s">
+      <c r="A2" s="66" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="64"/>
-      <c r="B3" s="62" t="s">
+      <c r="A3" s="66"/>
+      <c r="B3" s="64" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="62" t="s">
+      <c r="C3" s="64" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="64"/>
-      <c r="B4" s="62" t="s">
+      <c r="A4" s="66"/>
+      <c r="B4" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="62" t="s">
+      <c r="C4" s="64" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="62" t="s">
+      <c r="D4" s="64" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" ht="61" customHeight="1" spans="2:4">
-      <c r="B5" s="62" t="s">
+      <c r="B5" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="C5" s="62" t="s">
+      <c r="C5" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="65" t="s">
+      <c r="D5" s="67" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" ht="49" customHeight="1" spans="2:4">
-      <c r="B6" s="62" t="s">
+      <c r="B6" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="65" t="s">
+      <c r="C6" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="D6" s="65"/>
+      <c r="D6" s="67"/>
     </row>
     <row r="7" ht="71" customHeight="1" spans="2:4">
-      <c r="B7" s="62" t="s">
+      <c r="B7" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="48" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="65"/>
+      <c r="D7" s="67"/>
     </row>
     <row r="8" spans="2:4">
-      <c r="B8" s="62" t="s">
+      <c r="B8" s="64" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="62" t="s">
+      <c r="C8" s="64" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="65"/>
+      <c r="D8" s="67"/>
     </row>
     <row r="9" spans="2:3">
-      <c r="B9" s="62" t="s">
+      <c r="B9" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="62" t="s">
+      <c r="C9" s="64" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" ht="29" spans="2:3">
-      <c r="B10" s="62" t="s">
+    <row r="10" ht="30" spans="2:3">
+      <c r="B10" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="65" t="s">
+      <c r="C10" s="67" t="s">
         <v>36</v>
       </c>
     </row>
@@ -7070,13 +7046,13 @@
       <c r="C17" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E17" s="50" t="s">
+      <c r="E17" s="52" t="s">
         <v>41</v>
       </c>
-      <c r="F17" s="50"/>
-      <c r="G17" s="50"/>
-    </row>
-    <row r="18" s="2" customFormat="1" spans="2:5">
+      <c r="F17" s="52"/>
+      <c r="G17" s="52"/>
+    </row>
+    <row r="18" s="2" customFormat="1" ht="30" spans="2:5">
       <c r="B18" s="5" t="s">
         <v>9</v>
       </c>
@@ -7094,7 +7070,7 @@
       </c>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" s="2" customFormat="1" ht="29" spans="2:5">
+    <row r="20" s="2" customFormat="1" ht="30" spans="2:5">
       <c r="B20" s="5" t="s">
         <v>44</v>
       </c>
@@ -7112,10 +7088,10 @@
       <c r="C22"/>
     </row>
     <row r="23" hidden="1" spans="2:3">
-      <c r="B23" s="62" t="s">
+      <c r="B23" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="65" t="s">
+      <c r="C23" s="67" t="s">
         <v>46</v>
       </c>
     </row>
@@ -7135,14 +7111,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E65"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.1181818181818" customWidth="1"/>
-    <col min="2" max="2" width="39.1454545454545" style="13" customWidth="1"/>
-    <col min="3" max="3" width="61.5727272727273" style="13" customWidth="1"/>
-    <col min="4" max="4" width="66.8545454545455" style="13" customWidth="1"/>
-    <col min="5" max="5" width="64.5727272727273" style="13" customWidth="1"/>
-    <col min="6" max="256" width="11.8545454545455" customWidth="1"/>
+    <col min="1" max="1" width="13.1142857142857" customWidth="1"/>
+    <col min="2" max="2" width="39.1428571428571" style="13" customWidth="1"/>
+    <col min="3" max="3" width="61.5714285714286" style="13" customWidth="1"/>
+    <col min="4" max="4" width="66.8571428571429" style="13" customWidth="1"/>
+    <col min="5" max="5" width="64.5714285714286" style="13" customWidth="1"/>
+    <col min="6" max="256" width="11.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="19" customFormat="1" spans="1:5">
@@ -7200,7 +7176,7 @@
       </c>
       <c r="E5" s="25"/>
     </row>
-    <row r="6" spans="2:5">
+    <row r="6" ht="30" spans="2:5">
       <c r="B6" s="21" t="s">
         <v>27</v>
       </c>
@@ -7209,7 +7185,7 @@
       </c>
       <c r="E6" s="25"/>
     </row>
-    <row r="7" ht="58" spans="2:5">
+    <row r="7" ht="60" spans="2:5">
       <c r="B7" s="13" t="s">
         <v>51</v>
       </c>
@@ -7219,11 +7195,11 @@
       <c r="D7" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="50" t="s">
+      <c r="E7" s="52" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="8" ht="58" spans="2:5">
+    <row r="8" ht="60" spans="2:5">
       <c r="B8" s="13" t="s">
         <v>55</v>
       </c>
@@ -7239,7 +7215,7 @@
       <c r="B9" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="57" t="s">
+      <c r="C9" s="59" t="s">
         <v>59</v>
       </c>
       <c r="E9" s="25"/>
@@ -7280,7 +7256,7 @@
       </c>
       <c r="E12" s="25"/>
     </row>
-    <row r="13" ht="58" spans="2:5">
+    <row r="13" ht="60" spans="2:5">
       <c r="B13" s="13" t="s">
         <v>68</v>
       </c>
@@ -7292,7 +7268,7 @@
       </c>
       <c r="E13" s="25"/>
     </row>
-    <row r="14" ht="29" spans="2:5">
+    <row r="14" ht="30" spans="2:5">
       <c r="B14" s="13" t="s">
         <v>71</v>
       </c>
@@ -7328,7 +7304,7 @@
       </c>
       <c r="E16" s="25"/>
     </row>
-    <row r="17" ht="130.5" spans="2:5">
+    <row r="17" ht="135" spans="2:5">
       <c r="B17" s="13" t="s">
         <v>80</v>
       </c>
@@ -7385,14 +7361,14 @@
       </c>
       <c r="E22" s="25"/>
     </row>
-    <row r="23" ht="87" spans="2:5">
+    <row r="23" ht="90" spans="2:5">
       <c r="B23" s="13" t="s">
         <v>93</v>
       </c>
       <c r="C23" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="E23" s="46" t="s">
+      <c r="E23" s="50" t="s">
         <v>95</v>
       </c>
     </row>
@@ -7417,401 +7393,399 @@
       </c>
       <c r="E25" s="25"/>
     </row>
-    <row r="26" ht="87" spans="2:5">
+    <row r="26" ht="30" spans="2:5">
       <c r="B26" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="E26" s="46" t="s">
+      <c r="E26" s="47"/>
+    </row>
+    <row r="27" ht="45" spans="2:5">
+      <c r="B27" s="29" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="27" ht="29" spans="2:5">
-      <c r="B27" s="29" t="s">
+      <c r="C27" s="29" t="s">
         <v>104</v>
       </c>
-      <c r="C27" s="29" t="s">
+      <c r="D27" s="60" t="s">
         <v>105</v>
       </c>
-      <c r="D27" s="58" t="s">
+      <c r="E27" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="E27" s="8" t="s">
+    </row>
+    <row r="28" ht="30" spans="2:5">
+      <c r="B28" s="29" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="28" ht="29" spans="2:5">
-      <c r="B28" s="29" t="s">
+      <c r="C28" s="29" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="29" t="s">
+      <c r="D28" s="60"/>
+      <c r="E28" s="61"/>
+    </row>
+    <row r="29" ht="30" spans="2:5">
+      <c r="B29" s="29" t="s">
         <v>109</v>
       </c>
-      <c r="D28" s="58"/>
-      <c r="E28" s="59"/>
-    </row>
-    <row r="29" spans="2:5">
-      <c r="B29" s="29" t="s">
+      <c r="C29" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="C29" s="29" t="s">
+      <c r="D29" s="60"/>
+      <c r="E29" s="61"/>
+    </row>
+    <row r="30" ht="30" spans="2:5">
+      <c r="B30" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="D29" s="58"/>
-      <c r="E29" s="59"/>
-    </row>
-    <row r="30" ht="29" spans="2:5">
-      <c r="B30" s="29" t="s">
+      <c r="C30" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="C30" s="29" t="s">
-        <v>113</v>
-      </c>
-      <c r="D30" s="58"/>
-      <c r="E30" s="59"/>
+      <c r="D30" s="60"/>
+      <c r="E30" s="61"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="D31" s="60"/>
+      <c r="E31" s="8"/>
+    </row>
+    <row r="32" ht="30" spans="2:5">
+      <c r="B32" s="29" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32" s="60" t="s">
         <v>115</v>
       </c>
-      <c r="D31" s="58"/>
-      <c r="E31" s="8"/>
-    </row>
-    <row r="32" ht="29" spans="2:5">
-      <c r="B32" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="D32" s="58" t="s">
+      <c r="E32" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="E32" s="8" t="s">
+    </row>
+    <row r="33" ht="30" spans="2:5">
+      <c r="B33" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" s="29" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="33" ht="29" spans="2:5">
-      <c r="B33" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="C33" s="29" t="s">
+      <c r="D33" s="60"/>
+      <c r="E33" s="61"/>
+    </row>
+    <row r="34" ht="30" spans="2:5">
+      <c r="B34" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="D33" s="58"/>
-      <c r="E33" s="59"/>
-    </row>
-    <row r="34" spans="2:5">
-      <c r="B34" s="29" t="s">
-        <v>110</v>
-      </c>
-      <c r="C34" s="29" t="s">
-        <v>119</v>
-      </c>
-      <c r="D34" s="58"/>
-      <c r="E34" s="59"/>
-    </row>
-    <row r="35" ht="29" spans="2:5">
+      <c r="D34" s="60"/>
+      <c r="E34" s="61"/>
+    </row>
+    <row r="35" ht="30" spans="2:5">
       <c r="B35" s="29" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C35" s="29" t="s">
-        <v>118</v>
-      </c>
-      <c r="D35" s="58"/>
-      <c r="E35" s="59"/>
+        <v>117</v>
+      </c>
+      <c r="D35" s="60"/>
+      <c r="E35" s="61"/>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="29" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="D36" s="58"/>
-      <c r="E36" s="59"/>
+        <v>119</v>
+      </c>
+      <c r="D36" s="60"/>
+      <c r="E36" s="61"/>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="29" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C37" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D37" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="D37" s="58" t="s">
+      <c r="E37" s="61"/>
+    </row>
+    <row r="38" ht="45" spans="2:5">
+      <c r="B38" s="29" t="s">
         <v>122</v>
       </c>
-      <c r="E37" s="59"/>
-    </row>
-    <row r="38" ht="43.5" spans="2:5">
-      <c r="B38" s="29" t="s">
+      <c r="C38" s="29" t="s">
         <v>123</v>
       </c>
-      <c r="C38" s="29" t="s">
+      <c r="D38" s="60"/>
+      <c r="E38" s="69" t="s">
         <v>124</v>
       </c>
-      <c r="D38" s="58"/>
-      <c r="E38" s="67" t="s">
+    </row>
+    <row r="39" ht="135" spans="2:5">
+      <c r="B39" s="62" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="39" ht="130.5" spans="2:5">
-      <c r="B39" s="60" t="s">
+      <c r="C39" s="62"/>
+      <c r="D39" s="62" t="s">
         <v>126</v>
       </c>
-      <c r="C39" s="60"/>
-      <c r="D39" s="60" t="s">
+      <c r="E39" s="25" t="s">
         <v>127</v>
       </c>
-      <c r="E39" s="25" t="s">
+    </row>
+    <row r="40" ht="135" spans="2:5">
+      <c r="B40" s="62" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="40" ht="130.5" spans="2:5">
-      <c r="B40" s="60" t="s">
+      <c r="C40" s="62"/>
+      <c r="D40" s="62" t="s">
         <v>129</v>
       </c>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60" t="s">
-        <v>130</v>
-      </c>
       <c r="E40" s="25" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="41" spans="2:5">
       <c r="B41" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="C41" s="13" t="s">
         <v>131</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>132</v>
       </c>
       <c r="E41" s="25"/>
     </row>
     <row r="42" spans="2:5">
       <c r="B42" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="C42" s="26" t="s">
         <v>133</v>
-      </c>
-      <c r="C42" s="26" t="s">
-        <v>134</v>
       </c>
       <c r="E42" s="25"/>
     </row>
     <row r="43" spans="2:5">
       <c r="B43" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" s="13" t="s">
         <v>135</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>136</v>
       </c>
       <c r="E43" s="25"/>
     </row>
     <row r="44" spans="2:5">
       <c r="B44" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="C44" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="E44" s="25"/>
+    </row>
+    <row r="45" ht="195" spans="2:5">
+      <c r="B45" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C44" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="E44" s="25"/>
-    </row>
-    <row r="45" ht="188.5" spans="2:5">
-      <c r="B45" s="21" t="s">
+      <c r="C45" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="C45" s="13" t="s">
+      <c r="D45" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="E45" s="25"/>
+    </row>
+    <row r="46" ht="195" spans="2:5">
+      <c r="B46" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="E45" s="25"/>
-    </row>
-    <row r="46" ht="188.5" spans="2:5">
-      <c r="B46" s="21" t="s">
+      <c r="C46" s="13" t="s">
         <v>141</v>
       </c>
-      <c r="C46" s="13" t="s">
+      <c r="D46" s="57" t="s">
         <v>142</v>
       </c>
-      <c r="D46" s="55" t="s">
+      <c r="E46" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="E46" s="50" t="s">
+    </row>
+    <row r="47" ht="195" spans="2:5">
+      <c r="B47" s="21" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="47" ht="188.5" spans="2:5">
-      <c r="B47" s="21" t="s">
+      <c r="C47" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="C47" s="13" t="s">
+      <c r="D47" s="13" t="s">
         <v>146</v>
-      </c>
-      <c r="D47" s="13" t="s">
-        <v>147</v>
       </c>
       <c r="E47" s="25"/>
     </row>
     <row r="48" spans="2:5">
       <c r="B48" s="13" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E48" s="25"/>
     </row>
     <row r="49" spans="2:5">
       <c r="B49" s="13" t="s">
+        <v>148</v>
+      </c>
+      <c r="C49" s="26" t="s">
         <v>149</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>150</v>
       </c>
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="2:5">
       <c r="B50" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="C50" s="13" t="s">
         <v>151</v>
-      </c>
-      <c r="C50" s="13" t="s">
-        <v>152</v>
       </c>
       <c r="E50" s="25"/>
     </row>
     <row r="51" spans="2:5">
       <c r="B51" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E51" s="25"/>
+    </row>
+    <row r="52" ht="150" spans="2:5">
+      <c r="B52" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C51" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="E51" s="25"/>
-    </row>
-    <row r="52" ht="145" spans="2:5">
-      <c r="B52" s="13" t="s">
+      <c r="C52" s="14" t="s">
         <v>154</v>
       </c>
-      <c r="C52" s="14" t="s">
+      <c r="D52" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="E52" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="53" spans="2:5">
       <c r="B53" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="C53" s="26" t="s">
         <v>158</v>
-      </c>
-      <c r="C53" s="26" t="s">
-        <v>159</v>
       </c>
       <c r="E53" s="25"/>
     </row>
     <row r="54" spans="2:5">
       <c r="B54" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E54" s="25"/>
     </row>
     <row r="55" spans="2:5">
       <c r="B55" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C55" s="26" t="s">
         <v>161</v>
-      </c>
-      <c r="C55" s="26" t="s">
-        <v>162</v>
       </c>
       <c r="E55" s="25"/>
     </row>
     <row r="56" spans="2:5">
       <c r="B56" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C56" s="13" t="s">
         <v>163</v>
-      </c>
-      <c r="C56" s="13" t="s">
-        <v>164</v>
       </c>
       <c r="E56" s="25"/>
     </row>
     <row r="57" spans="2:5">
       <c r="B57" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E57" s="25"/>
     </row>
     <row r="58" spans="2:5">
       <c r="B58" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="C58" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="C58" s="26" t="s">
+      <c r="E58" s="25"/>
+    </row>
+    <row r="59" ht="180" spans="2:5">
+      <c r="B59" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E58" s="25"/>
-    </row>
-    <row r="59" ht="174" spans="2:5">
-      <c r="B59" s="13" t="s">
+      <c r="C59" s="26" t="s">
         <v>168</v>
       </c>
-      <c r="C59" s="26" t="s">
+      <c r="D59" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="D59" s="13" t="s">
+      <c r="E59" s="25"/>
+    </row>
+    <row r="60" ht="255" spans="2:5">
+      <c r="B60" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="E59" s="25"/>
-    </row>
-    <row r="60" ht="246.5" spans="2:5">
-      <c r="B60" s="13" t="s">
+      <c r="C60" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="C60" s="13" t="s">
+      <c r="D60" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="D60" s="13" t="s">
+      <c r="E60" s="25" t="s">
         <v>173</v>
-      </c>
-      <c r="E60" s="25" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="61" spans="2:5">
       <c r="B61" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C61" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="D61" s="63" t="s">
         <v>176</v>
-      </c>
-      <c r="D61" s="61" t="s">
-        <v>177</v>
       </c>
       <c r="E61" s="25"/>
     </row>
     <row r="62" ht="42.95" customHeight="1" spans="2:5">
       <c r="B62" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C62" s="59" t="s">
         <v>178</v>
       </c>
-      <c r="C62" s="57" t="s">
-        <v>179</v>
-      </c>
-      <c r="D62" s="61"/>
+      <c r="D62" s="63"/>
       <c r="E62" s="25"/>
     </row>
     <row r="65" spans="3:3">
-      <c r="C65" s="57"/>
+      <c r="C65" s="59"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -7835,14 +7809,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="9.14545454545454" customWidth="1"/>
-    <col min="2" max="2" width="40.8545454545455" customWidth="1"/>
-    <col min="3" max="3" width="61.5727272727273" customWidth="1"/>
-    <col min="4" max="4" width="57.4272727272727" customWidth="1"/>
-    <col min="5" max="5" width="54.8545454545455" customWidth="1"/>
-    <col min="6" max="6" width="9.14545454545454" customWidth="1"/>
+    <col min="1" max="1" width="9.14285714285714" customWidth="1"/>
+    <col min="2" max="2" width="40.8571428571429" customWidth="1"/>
+    <col min="3" max="3" width="61.5714285714286" customWidth="1"/>
+    <col min="4" max="4" width="57.4285714285714" customWidth="1"/>
+    <col min="5" max="5" width="54.8571428571429" customWidth="1"/>
+    <col min="6" max="6" width="9.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -7866,19 +7840,19 @@
       <c r="A2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="51" t="s">
-        <v>180</v>
-      </c>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
+      <c r="B2" s="53" t="s">
+        <v>179</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" s="13" t="s">
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E3" s="25"/>
     </row>
@@ -7896,7 +7870,7 @@
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E5" s="25"/>
     </row>
@@ -7905,206 +7879,206 @@
         <v>27</v>
       </c>
       <c r="C6" t="s">
+        <v>182</v>
+      </c>
+      <c r="E6" s="25"/>
+    </row>
+    <row r="7" ht="45" spans="2:5">
+      <c r="B7" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="E6" s="25"/>
-    </row>
-    <row r="7" ht="29" spans="2:5">
-      <c r="B7" s="20" t="s">
+      <c r="C7" t="s">
         <v>184</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>185</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" s="54" t="s">
         <v>186</v>
       </c>
-      <c r="E7" s="52" t="s">
+    </row>
+    <row r="8" ht="135" spans="2:5">
+      <c r="B8" s="55" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="8" ht="130.5" spans="2:5">
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="28" t="s">
         <v>188</v>
       </c>
-      <c r="C8" s="28" t="s">
+      <c r="D8" s="56" t="s">
         <v>189</v>
       </c>
-      <c r="D8" s="54" t="s">
+      <c r="E8" s="8" t="s">
         <v>190</v>
       </c>
-      <c r="E8" s="8" t="s">
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="55" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="9" spans="2:5">
-      <c r="B9" s="53" t="s">
+      <c r="C9" s="28" t="s">
         <v>192</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>193</v>
       </c>
       <c r="D9" s="28"/>
       <c r="E9" s="25"/>
     </row>
     <row r="10" spans="2:5">
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="55" t="s">
+        <v>193</v>
+      </c>
+      <c r="C10" s="28" t="s">
         <v>194</v>
-      </c>
-      <c r="C10" s="28" t="s">
-        <v>195</v>
       </c>
       <c r="D10" s="28"/>
       <c r="E10" s="25" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" ht="225" spans="2:5">
+      <c r="B11" s="20" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="11" ht="217.5" spans="2:5">
-      <c r="B11" s="20" t="s">
+      <c r="C11" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="57" t="s">
         <v>198</v>
       </c>
-      <c r="D11" s="55" t="s">
-        <v>199</v>
-      </c>
       <c r="E11" s="25" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="20" t="s">
+        <v>199</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>201</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="E13" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="14" ht="30" spans="2:5">
+      <c r="B14" s="20" t="s">
         <v>203</v>
       </c>
-      <c r="E13" s="8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="14" ht="29" spans="2:5">
-      <c r="B14" s="20" t="s">
+      <c r="C14" t="s">
         <v>204</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>205</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" s="25" t="s">
         <v>206</v>
       </c>
-      <c r="E14" s="25" t="s">
+    </row>
+    <row r="15" ht="135" spans="2:5">
+      <c r="B15" s="20" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="15" ht="116" spans="2:5">
-      <c r="B15" s="20" t="s">
+      <c r="C15" s="29" t="s">
         <v>208</v>
       </c>
-      <c r="C15" s="29" t="s">
+      <c r="D15" s="29" t="s">
         <v>209</v>
       </c>
-      <c r="D15" s="29" t="s">
+      <c r="E15" s="54" t="s">
         <v>210</v>
       </c>
-      <c r="E15" s="52" t="s">
+    </row>
+    <row r="16" ht="45" spans="2:5">
+      <c r="B16" s="20" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="16" ht="43.5" spans="2:5">
-      <c r="B16" s="20" t="s">
+      <c r="C16" s="2" t="s">
         <v>212</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="E16" s="25"/>
+    </row>
+    <row r="17" ht="60" spans="2:5">
+      <c r="B17" s="55" t="s">
         <v>214</v>
       </c>
-      <c r="E16" s="25"/>
-    </row>
-    <row r="17" ht="58" spans="2:5">
-      <c r="B17" s="53" t="s">
+      <c r="C17" s="58" t="s">
         <v>215</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="D17" s="29" t="s">
         <v>216</v>
       </c>
-      <c r="D17" s="29" t="s">
+      <c r="E17" s="25"/>
+    </row>
+    <row r="18" ht="60" spans="2:5">
+      <c r="B18" s="58" t="s">
         <v>217</v>
       </c>
-      <c r="E17" s="25"/>
-    </row>
-    <row r="18" ht="58" spans="2:5">
-      <c r="B18" s="56" t="s">
+      <c r="C18" s="58" t="s">
         <v>218</v>
       </c>
-      <c r="C18" s="56" t="s">
+      <c r="D18" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>220</v>
-      </c>
       <c r="E18" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="29" t="s">
         <v>222</v>
       </c>
-      <c r="D19" s="29" t="s">
-        <v>223</v>
-      </c>
       <c r="E19" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>224</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>225</v>
       </c>
       <c r="D20" s="29"/>
       <c r="E20" s="8" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" ht="77" customHeight="1" spans="2:5">
       <c r="B21" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C21" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D21" s="13" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E21" s="25"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D22" s="13"/>
       <c r="E22" s="25"/>
@@ -8124,14 +8098,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="43.5727272727273" customWidth="1"/>
-    <col min="5" max="5" width="57.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="9.14545454545454" customWidth="1"/>
+    <col min="4" max="4" width="43.5714285714286" customWidth="1"/>
+    <col min="5" max="5" width="57.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="9.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8162,7 +8136,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="25"/>
     </row>
@@ -8175,7 +8149,7 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="E4" s="25"/>
     </row>
@@ -8190,270 +8164,270 @@
       <c r="D5" s="13"/>
       <c r="E5" s="25"/>
     </row>
-    <row r="6" ht="29" spans="2:5">
+    <row r="6" ht="30" spans="2:5">
       <c r="B6" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="25"/>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C7" s="13"/>
       <c r="D7" t="s">
+        <v>230</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" ht="75" spans="2:5">
+      <c r="B8" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="E7" s="8" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="8" ht="72.5" spans="2:5">
-      <c r="B8" s="20" t="s">
+      <c r="C8" s="51" t="s">
         <v>232</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="D8" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="E8" s="70" t="s">
         <v>234</v>
-      </c>
-      <c r="E8" s="68" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="20" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="51" t="s">
         <v>236</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>237</v>
       </c>
       <c r="D9" s="13"/>
       <c r="E9" s="25"/>
     </row>
-    <row r="10" ht="72.5" spans="2:5">
+    <row r="10" ht="75" spans="2:5">
       <c r="B10" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="C10" s="51" t="s">
         <v>238</v>
       </c>
-      <c r="C10" s="49" t="s">
+      <c r="D10" s="13"/>
+      <c r="E10" s="70" t="s">
         <v>239</v>
       </c>
-      <c r="D10" s="13"/>
-      <c r="E10" s="68" t="s">
+    </row>
+    <row r="11" ht="120" spans="2:5">
+      <c r="B11" s="20" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="11" ht="116" spans="2:5">
-      <c r="B11" s="20" t="s">
+      <c r="C11" s="14" t="s">
         <v>241</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="E11" s="52" t="s">
         <v>243</v>
       </c>
-      <c r="E11" s="50" t="s">
+    </row>
+    <row r="12" ht="60" spans="2:5">
+      <c r="B12" s="20" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="12" ht="43.5" spans="2:5">
-      <c r="B12" s="20" t="s">
+      <c r="E12" s="47" t="s">
         <v>245</v>
-      </c>
-      <c r="E12" s="46" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="13" spans="2:5">
       <c r="B13" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>247</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>248</v>
       </c>
       <c r="E13" s="25"/>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" t="s">
+        <v>248</v>
+      </c>
+      <c r="C14" t="s">
         <v>249</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" s="25"/>
+    </row>
+    <row r="15" ht="75" spans="2:5">
+      <c r="B15" s="20" t="s">
         <v>250</v>
       </c>
-      <c r="E14" s="25"/>
-    </row>
-    <row r="15" ht="72.5" spans="2:5">
-      <c r="B15" s="20" t="s">
+      <c r="C15" t="s">
         <v>251</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="E15" s="25"/>
+    </row>
+    <row r="16" ht="30" spans="2:5">
+      <c r="B16" s="20" t="s">
         <v>253</v>
       </c>
-      <c r="E15" s="25"/>
-    </row>
-    <row r="16" ht="29" spans="2:5">
-      <c r="B16" s="20" t="s">
+      <c r="C16" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="E16" s="25"/>
+    </row>
+    <row r="17" ht="60" spans="2:5">
+      <c r="B17" t="s">
         <v>255</v>
       </c>
-      <c r="E16" s="25"/>
-    </row>
-    <row r="17" ht="58" spans="2:5">
-      <c r="B17" t="s">
+      <c r="C17" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="D17" s="13" t="s">
         <v>257</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>258</v>
       </c>
       <c r="E17" s="25"/>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" t="s">
+        <v>258</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="E18" s="25"/>
+    </row>
+    <row r="19" ht="30" spans="2:5">
+      <c r="B19" t="s">
         <v>260</v>
       </c>
-      <c r="E18" s="25"/>
-    </row>
-    <row r="19" ht="29" spans="2:5">
-      <c r="B19" t="s">
+      <c r="C19" s="13" t="s">
         <v>261</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="D19" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="E19" s="25" t="s">
         <v>263</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" t="s">
+        <v>264</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>265</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>266</v>
       </c>
       <c r="D20" s="13"/>
       <c r="E20" s="25" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" t="s">
+        <v>267</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>268</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>269</v>
       </c>
       <c r="D21" s="13"/>
       <c r="E21" s="25" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="25" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="23" ht="29" spans="2:5">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="23" ht="30" spans="2:5">
       <c r="B23" t="s">
+        <v>270</v>
+      </c>
+      <c r="C23" s="13" t="s">
         <v>271</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>272</v>
       </c>
       <c r="D23" s="13"/>
       <c r="E23" s="25" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="24" ht="72.5" spans="2:5">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="24" ht="75" spans="2:5">
       <c r="B24" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C24" s="13"/>
       <c r="D24" s="13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="E24" s="25"/>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" t="s">
+        <v>274</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>275</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>276</v>
       </c>
       <c r="D25" s="13"/>
       <c r="E25" s="25"/>
     </row>
-    <row r="26" ht="58" spans="2:5">
+    <row r="26" ht="60" spans="2:5">
       <c r="B26" t="s">
+        <v>276</v>
+      </c>
+      <c r="C26" s="13" t="s">
         <v>277</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="D26" s="13" t="s">
         <v>278</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="E26" s="25" t="s">
         <v>279</v>
-      </c>
-      <c r="E26" s="25" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" t="s">
+        <v>280</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>281</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>282</v>
       </c>
       <c r="D27" s="13"/>
       <c r="E27" s="25" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" spans="2:5">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="28" customHeight="1" spans="2:5">
       <c r="B28" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D28" s="13" t="s">
+        <v>282</v>
+      </c>
+      <c r="E28" s="25"/>
+    </row>
+    <row r="29" ht="30" spans="2:5">
+      <c r="B29" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C29" s="13" t="s">
         <v>283</v>
-      </c>
-      <c r="E28" s="25"/>
-    </row>
-    <row r="29" ht="29" spans="2:5">
-      <c r="B29" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>284</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="25"/>
@@ -8473,15 +8447,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F31"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="19.4272727272727" style="31" customWidth="1"/>
+    <col min="1" max="1" width="19.4285714285714" style="31" customWidth="1"/>
     <col min="2" max="2" width="37" style="31" customWidth="1"/>
-    <col min="3" max="3" width="50.5727272727273" style="31" customWidth="1"/>
-    <col min="4" max="4" width="39.1454545454545" style="31" customWidth="1"/>
-    <col min="5" max="5" width="54.1454545454545" style="31" customWidth="1"/>
-    <col min="6" max="6" width="51.1454545454545" style="31" customWidth="1"/>
-    <col min="7" max="16384" width="9.14545454545454" style="31"/>
+    <col min="3" max="3" width="50.5714285714286" style="31" customWidth="1"/>
+    <col min="4" max="4" width="39.1428571428571" style="31" customWidth="1"/>
+    <col min="5" max="5" width="54.1428571428571" style="31" customWidth="1"/>
+    <col min="6" max="6" width="51.1428571428571" style="31" customWidth="1"/>
+    <col min="7" max="16384" width="9.14285714285714" style="31"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -8501,7 +8475,7 @@
         <v>17</v>
       </c>
       <c r="F1" s="33" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -8515,7 +8489,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="35" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E3" s="34"/>
     </row>
@@ -8539,231 +8513,228 @@
       <c r="D5" s="35"/>
       <c r="E5" s="34"/>
     </row>
-    <row r="6" ht="29" spans="2:5">
+    <row r="6" ht="30" spans="2:5">
       <c r="B6" s="35" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D6" s="35"/>
       <c r="E6" s="34"/>
     </row>
-    <row r="7" ht="29" spans="2:6">
+    <row r="7" ht="30" spans="2:6">
       <c r="B7" s="36" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C7" s="37"/>
       <c r="D7" s="37" t="s">
+        <v>288</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>289</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="F7" s="38"/>
+    </row>
+    <row r="8" ht="195" spans="2:5">
+      <c r="B8" s="31" t="s">
         <v>290</v>
       </c>
-      <c r="F7" s="38"/>
-    </row>
-    <row r="8" ht="188.5" spans="2:5">
-      <c r="B8" s="31" t="s">
+      <c r="C8" s="39" t="s">
         <v>291</v>
       </c>
-      <c r="C8" s="39" t="s">
+      <c r="D8" s="35" t="s">
         <v>292</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="E8" s="14" t="s">
         <v>293</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" s="31" t="s">
+        <v>294</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>295</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>296</v>
       </c>
       <c r="D9" s="35"/>
       <c r="E9" s="34"/>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="35" t="s">
+        <v>296</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>297</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>298</v>
       </c>
       <c r="D10" s="35"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="2:5">
+    <row r="11" ht="30" spans="2:5">
       <c r="B11" s="35" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D11" s="35"/>
       <c r="E11" s="34"/>
     </row>
-    <row r="12" spans="2:5">
+    <row r="12" ht="30" spans="2:5">
       <c r="B12" s="35" t="s">
+        <v>299</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>300</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>301</v>
       </c>
       <c r="D12" s="35"/>
       <c r="E12" s="34"/>
     </row>
-    <row r="13" ht="217.5" spans="2:5">
+    <row r="13" ht="225" spans="2:5">
       <c r="B13" s="31" t="s">
+        <v>301</v>
+      </c>
+      <c r="C13" s="39" t="s">
         <v>302</v>
       </c>
-      <c r="C13" s="39" t="s">
+      <c r="D13" s="35" t="s">
         <v>303</v>
       </c>
-      <c r="D13" s="35" t="s">
+      <c r="E13" s="40" t="s">
         <v>304</v>
-      </c>
-      <c r="E13" s="40" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="14" spans="2:5">
       <c r="B14" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>306</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>307</v>
       </c>
       <c r="D14" s="35"/>
       <c r="E14" s="34"/>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>309</v>
       </c>
       <c r="D15" s="35"/>
       <c r="E15" s="34"/>
     </row>
-    <row r="16" spans="2:5">
+    <row r="16" ht="30" spans="2:5">
       <c r="B16" s="35" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D16" s="35"/>
       <c r="E16" s="34"/>
     </row>
-    <row r="17" spans="2:5">
+    <row r="17" ht="30" spans="2:5">
       <c r="B17" s="35" t="s">
+        <v>310</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>311</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>312</v>
       </c>
       <c r="D17" s="35"/>
       <c r="E17" s="34"/>
     </row>
-    <row r="18" ht="29" spans="2:5">
+    <row r="18" ht="30" spans="2:5">
       <c r="B18" s="41" t="s">
+        <v>312</v>
+      </c>
+      <c r="C18" s="42" t="s">
         <v>313</v>
       </c>
-      <c r="C18" s="42" t="s">
+      <c r="D18" s="35" t="s">
         <v>314</v>
       </c>
-      <c r="D18" s="35" t="s">
+      <c r="E18" s="40" t="s">
         <v>315</v>
       </c>
-      <c r="E18" s="40" t="s">
+    </row>
+    <row r="19" ht="135" spans="2:5">
+      <c r="B19" s="37" t="s">
         <v>316</v>
-      </c>
-    </row>
-    <row r="19" ht="130.5" spans="2:5">
-      <c r="B19" s="37" t="s">
-        <v>317</v>
       </c>
       <c r="C19" s="43"/>
       <c r="D19" s="44" t="s">
+        <v>317</v>
+      </c>
+      <c r="E19" s="34" t="s">
         <v>318</v>
       </c>
-      <c r="E19" s="34" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="20" ht="58" spans="2:5">
+    </row>
+    <row r="20" ht="60" spans="2:5">
       <c r="B20" s="35" t="s">
         <v>96</v>
       </c>
       <c r="C20" s="45" t="s">
+        <v>319</v>
+      </c>
+      <c r="D20" s="35"/>
+      <c r="E20" s="71" t="s">
         <v>320</v>
       </c>
-      <c r="D20" s="35"/>
-      <c r="E20" s="69" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="21" ht="174" spans="2:5">
+    </row>
+    <row r="21" ht="180" spans="2:5">
       <c r="B21" s="35" t="s">
         <v>99</v>
       </c>
       <c r="C21" s="45" t="s">
+        <v>321</v>
+      </c>
+      <c r="D21" s="35" t="s">
         <v>322</v>
       </c>
-      <c r="D21" s="35" t="s">
-        <v>323</v>
-      </c>
       <c r="E21" s="34"/>
     </row>
-    <row r="22" ht="87" spans="2:6">
+    <row r="22" spans="2:6">
       <c r="B22" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="C22" s="45" t="s">
-        <v>324</v>
+      <c r="C22" s="46" t="s">
+        <v>323</v>
       </c>
       <c r="D22" s="35"/>
-      <c r="E22" s="46" t="s">
-        <v>325</v>
-      </c>
-      <c r="F22" s="47"/>
-    </row>
-    <row r="23" ht="29" spans="2:5">
+      <c r="E22" s="47"/>
+      <c r="F22" s="48"/>
+    </row>
+    <row r="23" ht="30" spans="2:5">
       <c r="B23" s="35" t="s">
         <v>80</v>
       </c>
-      <c r="C23" s="48" t="s">
-        <v>326</v>
+      <c r="C23" s="49" t="s">
+        <v>324</v>
       </c>
       <c r="D23" s="35" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="E23" s="34"/>
     </row>
-    <row r="24" ht="87" spans="2:6">
+    <row r="24" ht="90" spans="2:5">
       <c r="B24" s="35" t="s">
         <v>93</v>
       </c>
       <c r="C24" s="45" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D24" s="35"/>
-      <c r="E24" s="46" t="s">
-        <v>329</v>
-      </c>
-      <c r="F24" s="47"/>
-    </row>
-    <row r="25" ht="43.5" spans="2:5">
+      <c r="E24" s="50" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="25" ht="45" spans="2:5">
       <c r="B25" s="35" t="s">
         <v>83</v>
       </c>
-      <c r="C25" s="48" t="s">
-        <v>330</v>
+      <c r="C25" s="49" t="s">
+        <v>328</v>
       </c>
       <c r="D25" s="35"/>
       <c r="E25" s="34"/>
@@ -8773,7 +8744,7 @@
         <v>85</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D26" s="35"/>
       <c r="E26" s="34"/>
@@ -8783,7 +8754,7 @@
         <v>87</v>
       </c>
       <c r="C27" s="45" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D27" s="35"/>
       <c r="E27" s="34"/>
@@ -8793,7 +8764,7 @@
         <v>89</v>
       </c>
       <c r="C28" s="45" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="D28" s="35"/>
       <c r="E28" s="34"/>
@@ -8803,29 +8774,29 @@
         <v>91</v>
       </c>
       <c r="C29" s="45" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D29" s="35"/>
       <c r="E29" s="34"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="2:5">
+    <row r="30" customHeight="1" spans="2:5">
       <c r="B30" s="35" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" s="45" t="s">
         <v>175</v>
       </c>
-      <c r="C30" s="45" t="s">
-        <v>176</v>
-      </c>
       <c r="D30" s="35" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="E30" s="34"/>
     </row>
-    <row r="31" ht="29" spans="2:5">
+    <row r="31" ht="30" spans="2:5">
       <c r="B31" s="35" t="s">
-        <v>178</v>
-      </c>
-      <c r="C31" s="48" t="s">
-        <v>336</v>
+        <v>177</v>
+      </c>
+      <c r="C31" s="49" t="s">
+        <v>334</v>
       </c>
       <c r="D31" s="35"/>
       <c r="E31" s="34"/>
@@ -8835,9 +8806,6 @@
     <mergeCell ref="D23:D29"/>
     <mergeCell ref="D30:D31"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="C22" r:id="rId1" display="ORC.23.2" tooltip="https://hl7-definition.caristix.com/v2/HL7v2.7.1/Fields/ORC.23.2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
 </worksheet>
@@ -8847,14 +8815,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E28"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.2181818181818" customWidth="1"/>
-    <col min="2" max="2" width="26.2818181818182" customWidth="1"/>
-    <col min="3" max="3" width="43.7181818181818" customWidth="1"/>
-    <col min="4" max="4" width="47.2818181818182" customWidth="1"/>
-    <col min="5" max="5" width="80.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="9.14545454545454" customWidth="1"/>
+    <col min="1" max="1" width="13.2190476190476" customWidth="1"/>
+    <col min="2" max="2" width="26.2857142857143" customWidth="1"/>
+    <col min="3" max="3" width="43.7142857142857" customWidth="1"/>
+    <col min="4" max="4" width="47.2857142857143" customWidth="1"/>
+    <col min="5" max="5" width="80.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="9.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -8885,7 +8853,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E3" s="13"/>
     </row>
@@ -8897,7 +8865,7 @@
         <v>22</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="E4" s="13"/>
     </row>
@@ -8910,12 +8878,12 @@
       </c>
       <c r="E5" s="13"/>
     </row>
-    <row r="6" ht="29" spans="2:5">
+    <row r="6" ht="30" spans="2:5">
       <c r="B6" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="E6" s="13"/>
     </row>
@@ -8928,245 +8896,245 @@
         <v>53</v>
       </c>
       <c r="E7" s="22" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="8" ht="74.25" spans="2:5">
+      <c r="B8" s="21" t="s">
+        <v>183</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>340</v>
       </c>
-    </row>
-    <row r="8" ht="71.5" spans="2:5">
-      <c r="B8" s="21" t="s">
-        <v>184</v>
-      </c>
-      <c r="C8" s="13" t="s">
+      <c r="E8" s="10" t="s">
         <v>341</v>
       </c>
-      <c r="D8" s="13" t="s">
+    </row>
+    <row r="9" ht="120" spans="2:5">
+      <c r="B9" s="27" t="s">
         <v>342</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="9" ht="116" spans="2:5">
-      <c r="B9" s="27" t="s">
-        <v>344</v>
       </c>
       <c r="C9" s="28"/>
       <c r="D9" s="29" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="10" ht="43.5" spans="1:5">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="10" ht="45" spans="1:5">
       <c r="A10" s="28"/>
       <c r="B10" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D10" s="29"/>
       <c r="E10" s="8" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="11" ht="203" spans="1:5">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="11" ht="210" spans="1:5">
       <c r="A11" s="28"/>
       <c r="B11" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="29"/>
       <c r="E11" s="11" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="12" ht="203" spans="1:5">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" ht="210" spans="1:5">
       <c r="A12" s="28"/>
       <c r="B12" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="29"/>
       <c r="E12" s="11" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="28"/>
       <c r="B13" s="6" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="29"/>
       <c r="E13" s="8" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" ht="150" spans="2:5">
+      <c r="B14" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="C14" s="13" t="s">
         <v>352</v>
       </c>
-    </row>
-    <row r="14" ht="130.5" spans="2:5">
-      <c r="B14" s="13" t="s">
+      <c r="D14" s="13" t="s">
         <v>353</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>354</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>355</v>
       </c>
       <c r="E14" s="13"/>
     </row>
     <row r="15" spans="2:5">
       <c r="B15" s="21" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="E15" s="13"/>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="21" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E16" s="13"/>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="13" t="s">
+        <v>357</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>358</v>
+      </c>
+      <c r="E17" s="13"/>
+    </row>
+    <row r="18" ht="105" spans="2:5">
+      <c r="B18" s="13" t="s">
         <v>359</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C18" s="13" t="s">
         <v>360</v>
       </c>
-      <c r="E17" s="13"/>
-    </row>
-    <row r="18" ht="101.5" spans="2:5">
-      <c r="B18" s="13" t="s">
+      <c r="D18" s="13" t="s">
         <v>361</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="E18" s="13" t="s">
         <v>362</v>
       </c>
-      <c r="D18" s="13" t="s">
+    </row>
+    <row r="19" ht="30" spans="2:5">
+      <c r="B19" s="13" t="s">
         <v>363</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="C19" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="20" ht="30" spans="2:5">
+      <c r="B20" s="13" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="19" ht="29" spans="2:5">
-      <c r="B19" s="13" t="s">
+      <c r="C20" s="13" t="s">
+        <v>360</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="21" ht="75" spans="2:5">
+      <c r="B21" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>365</v>
       </c>
-      <c r="C19" s="13" t="s">
-        <v>362</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="20" ht="29" spans="2:5">
-      <c r="B20" s="13" t="s">
+      <c r="D21" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="C20" s="13" t="s">
-        <v>362</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="21" ht="72.5" spans="2:5">
-      <c r="B21" s="21" t="s">
-        <v>251</v>
-      </c>
-      <c r="C21" s="12" t="s">
+      <c r="E21" s="13"/>
+    </row>
+    <row r="22" ht="30" spans="2:5">
+      <c r="B22" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="E22" s="13"/>
+    </row>
+    <row r="23" ht="45" spans="2:5">
+      <c r="B23" s="27" t="s">
         <v>367</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="C23" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="E21" s="13"/>
-    </row>
-    <row r="22" ht="29" spans="2:5">
-      <c r="B22" s="21" t="s">
-        <v>254</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>255</v>
-      </c>
-      <c r="E22" s="13"/>
-    </row>
-    <row r="23" ht="43.5" spans="2:5">
-      <c r="B23" s="27" t="s">
+      <c r="D23" s="29" t="s">
         <v>369</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="E23" s="13"/>
+    </row>
+    <row r="24" ht="30" spans="2:5">
+      <c r="B24" s="21" t="s">
         <v>370</v>
       </c>
-      <c r="D23" s="29" t="s">
+      <c r="C24" s="13" t="s">
         <v>371</v>
       </c>
-      <c r="E23" s="13"/>
-    </row>
-    <row r="24" spans="2:5">
-      <c r="B24" s="21" t="s">
+      <c r="D24" s="13" t="s">
         <v>372</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="E24" s="13" t="s">
         <v>373</v>
       </c>
-      <c r="D24" s="13" t="s">
+    </row>
+    <row r="25" ht="60" spans="2:5">
+      <c r="B25" s="13" t="s">
         <v>374</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="C25" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="D25" s="13" t="s">
         <v>375</v>
       </c>
-    </row>
-    <row r="25" ht="58" spans="2:5">
-      <c r="B25" s="13" t="s">
+      <c r="E25" s="13"/>
+    </row>
+    <row r="26" ht="30" spans="2:5">
+      <c r="B26" s="13" t="s">
         <v>376</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="D25" s="13" t="s">
+      <c r="C26" s="13" t="s">
         <v>377</v>
       </c>
-      <c r="E25" s="13"/>
-    </row>
-    <row r="26" ht="29" spans="2:5">
-      <c r="B26" s="13" t="s">
+      <c r="D26" s="13" t="s">
         <v>378</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>379</v>
-      </c>
-      <c r="D26" s="13" t="s">
-        <v>380</v>
       </c>
       <c r="E26" s="13"/>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>176</v>
-      </c>
       <c r="D27" s="13" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="E27" s="13"/>
     </row>
     <row r="28" ht="78" customHeight="1" spans="2:5">
       <c r="B28" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D28" s="13"/>
       <c r="E28" s="13"/>
@@ -9192,14 +9160,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="22.2818181818182" customWidth="1"/>
+    <col min="1" max="1" width="22.2857142857143" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="70.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="47.1454545454545" customWidth="1"/>
-    <col min="5" max="5" width="49.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="9.14545454545454" customWidth="1"/>
+    <col min="3" max="3" width="70.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="47.1428571428571" customWidth="1"/>
+    <col min="5" max="5" width="49.5714285714286" customWidth="1"/>
+    <col min="6" max="6" width="9.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9219,9 +9187,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" ht="29" spans="1:5">
+    <row r="2" ht="30" spans="1:5">
       <c r="A2" s="24" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="E2" s="25"/>
     </row>
@@ -9231,7 +9199,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E3" s="25"/>
     </row>
@@ -9244,7 +9212,7 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="E4" s="25"/>
     </row>
@@ -9259,157 +9227,157 @@
       <c r="D5" s="13"/>
       <c r="E5" s="25"/>
     </row>
-    <row r="6" ht="29" spans="2:5">
+    <row r="6" ht="30" spans="2:5">
       <c r="B6" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="25"/>
     </row>
-    <row r="7" ht="71.5" spans="2:5">
+    <row r="7" ht="74.25" spans="2:5">
       <c r="B7" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="D7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
     </row>
     <row r="8" spans="2:5">
       <c r="B8" s="20" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C8" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="25"/>
     </row>
     <row r="9" ht="42.95" customHeight="1" spans="2:5">
       <c r="B9" s="20" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C9" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="E9" s="25"/>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" s="20" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D10" s="13"/>
       <c r="E10" s="25"/>
     </row>
     <row r="11" ht="60.95" customHeight="1" spans="2:5">
       <c r="B11" s="20" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="D11" s="13"/>
       <c r="E11" s="25"/>
     </row>
-    <row r="12" ht="29" spans="2:5">
+    <row r="12" ht="30" spans="2:5">
       <c r="B12" s="13" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>389</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="E12" s="25"/>
+    </row>
+    <row r="13" ht="30" spans="2:5">
+      <c r="B13" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>391</v>
-      </c>
-      <c r="D12" s="13" t="s">
-        <v>392</v>
-      </c>
-      <c r="E12" s="25"/>
-    </row>
-    <row r="13" ht="29" spans="2:5">
-      <c r="B13" s="13" t="s">
-        <v>365</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>393</v>
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="25"/>
     </row>
     <row r="14" ht="78" customHeight="1" spans="2:5">
       <c r="B14" s="13" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="D14" s="13"/>
       <c r="E14" s="25"/>
     </row>
-    <row r="15" ht="43.5" spans="2:5">
+    <row r="15" ht="45" spans="2:5">
       <c r="B15" s="20" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="E15" s="25"/>
     </row>
     <row r="16" spans="2:5">
       <c r="B16" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>255</v>
-      </c>
       <c r="E16" s="25"/>
     </row>
-    <row r="17" ht="29" spans="2:5">
+    <row r="17" ht="30" spans="2:5">
       <c r="B17" t="s">
+        <v>370</v>
+      </c>
+      <c r="C17" t="s">
+        <v>394</v>
+      </c>
+      <c r="D17" t="s">
         <v>372</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" s="25" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="18" customHeight="1" spans="2:5">
+      <c r="B18" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="D18" s="13" t="s">
         <v>396</v>
-      </c>
-      <c r="D17" t="s">
-        <v>374</v>
-      </c>
-      <c r="E17" s="25" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" spans="2:5">
-      <c r="B18" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>398</v>
       </c>
       <c r="E18" s="25"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="13" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="D19" s="13"/>
       <c r="E19" s="25"/>
@@ -9429,14 +9397,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr defaultColWidth="9.14545454545454" defaultRowHeight="14.5" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="9.14545454545454" customWidth="1"/>
-    <col min="2" max="2" width="23.1454545454545" customWidth="1"/>
-    <col min="3" max="3" width="34.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="25.1454545454545" customWidth="1"/>
-    <col min="5" max="5" width="33.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="9.14545454545454" customWidth="1"/>
+    <col min="1" max="1" width="9.14285714285714" customWidth="1"/>
+    <col min="2" max="2" width="23.1428571428571" customWidth="1"/>
+    <col min="3" max="3" width="34.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="25.1428571428571" customWidth="1"/>
+    <col min="5" max="5" width="33.4285714285714" customWidth="1"/>
+    <col min="6" max="6" width="9.14285714285714" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -9466,7 +9434,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9478,7 +9446,7 @@
         <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -9492,130 +9460,130 @@
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
     </row>
-    <row r="6" ht="29" spans="2:5">
+    <row r="6" ht="45" spans="2:5">
       <c r="B6" s="21" t="s">
         <v>27</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" s="20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C7" s="13" t="s">
+        <v>400</v>
+      </c>
+      <c r="D7" t="s">
+        <v>401</v>
+      </c>
+      <c r="E7" s="22"/>
+    </row>
+    <row r="8" ht="165" spans="2:5">
+      <c r="B8" s="20" t="s">
+        <v>351</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>402</v>
       </c>
-      <c r="D7" t="s">
-        <v>403</v>
-      </c>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="8" ht="159.5" spans="2:5">
-      <c r="B8" s="20" t="s">
-        <v>353</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>404</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E8" s="23"/>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="20" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="20" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11" spans="2:3">
       <c r="B11" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C11" s="13" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="12" ht="90" spans="2:4">
+      <c r="B12" s="20" t="s">
+        <v>250</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>406</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="13" ht="45" spans="2:3">
+      <c r="B13" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="14" ht="75" spans="2:4">
+      <c r="B14" s="20" t="s">
+        <v>367</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>368</v>
+      </c>
+      <c r="D14" s="13" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="12" ht="87" spans="2:4">
-      <c r="B12" s="20" t="s">
-        <v>251</v>
-      </c>
-      <c r="C12" s="13" t="s">
+    <row r="15" ht="90" spans="2:4">
+      <c r="B15" t="s">
         <v>408</v>
       </c>
-      <c r="D12" s="13" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="13" ht="29" spans="2:3">
-      <c r="B13" s="20" t="s">
-        <v>254</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="14" ht="72.5" spans="2:4">
-      <c r="B14" s="20" t="s">
-        <v>369</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>370</v>
-      </c>
-      <c r="D14" s="13" t="s">
+      <c r="C15" s="13" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="15" ht="87" spans="2:4">
-      <c r="B15" t="s">
+      <c r="D15" s="13" t="s">
         <v>410</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>411</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="16" spans="2:3">
       <c r="B16" t="s">
+        <v>411</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="17" customHeight="1" spans="2:4">
+      <c r="B17" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="D17" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="C16" s="13" t="s">
+    </row>
+    <row r="18" ht="30" spans="2:4">
+      <c r="B18" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>414</v>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" spans="2:4">
-      <c r="B17" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="18" ht="29" spans="2:4">
-      <c r="B18" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>416</v>
       </c>
       <c r="D18" s="13"/>
     </row>

</xml_diff>

<commit_message>
feat: update HL7 to FHIR conversion specification document with latest changes
</commit_message>
<xml_diff>
--- a/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
+++ b/support/specifications/hl7/HL7v2.to.FHIR.Conversion.Spec.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="753" firstSheet="1" activeTab="6"/>
+    <workbookView windowWidth="28800" windowHeight="12180" tabRatio="753" firstSheet="1" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="477">
   <si>
     <t>FHIR Resources</t>
   </si>
@@ -1890,6 +1890,107 @@
     <t>The HL7 file shared does not contain the NK1 segment.</t>
   </si>
   <si>
+    <t>maritalStatus -&gt; coding -&gt; system</t>
+  </si>
+  <si>
+    <t>If maritalStatus code is "UNK" then "http://terminology.hl7.org/CodeSystem/v3-NullFlavor", otherwise "http://terminology.hl7.org/CodeSystem/v3-MaritalStatus".</t>
+  </si>
+  <si>
+    <t>maritalStatus -&gt; coding -&gt; code</t>
+  </si>
+  <si>
+    <t>PID.16.1</t>
+  </si>
+  <si>
+    <t>maritalStatus -&gt; coding -&gt; display</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>maritalStatusCode.code -&gt;  maritalStatus.display Mapping</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+M -&gt; married  
+S -&gt; never married  
+A -&gt; annulled  
+D -&gt; divorced  
+I -&gt; interlocutory  
+L -&gt; legally separated  
+C -&gt; common law  
+P -&gt; polygamous  
+T -&gt; domestic partner  
+U -&gt; unmarried  
+W -&gt; widowed  
+All Others -&gt; unknown</t>
+    </r>
+  </si>
+  <si>
+    <t>deceasedBoolean</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If PID.30.1 is "Y" then </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>true</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> else </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>false</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
     <t>request -&gt; method</t>
   </si>
   <si>
@@ -4347,6 +4448,14 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Question Code -&gt; Category Display Mapping</t>
     </r>
     <r>
@@ -4605,6 +4714,15 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+        <scheme val="minor"/>
+      </rPr>
       <t>Interpretation Code -&gt; Interpretation Display Mapping</t>
     </r>
     <r>
@@ -5823,6 +5941,36 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color indexed="10"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -5836,42 +5984,12 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="40">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5888,12 +6006,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
         <bgColor rgb="FFE7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -6239,7 +6351,7 @@
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -6263,16 +6375,16 @@
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="35" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="36" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -6281,100 +6393,100 @@
     <xf numFmtId="0" fontId="38" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="39" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="40" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="41" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="42" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="43" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="42" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="44" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="45" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="45" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="45" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="44" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="44" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="46" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="47" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0">
@@ -6396,7 +6508,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -6511,10 +6623,10 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -6532,11 +6644,14 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
@@ -6574,6 +6689,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -6583,7 +6701,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -6680,7 +6810,7 @@
     <cellStyle name="Warning" xfId="59"/>
   </cellStyles>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{58ECC587-4D15-4AA1-90CF-3197D7A288C3}"/>
+    <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{A0F109D3-22A3-4D89-8C49-8EB962CB3793}"/>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -6951,66 +7081,66 @@
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultColWidth="11.8571428571429" defaultRowHeight="15" outlineLevelRow="7" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="14.2857142857143" style="70" customWidth="1"/>
+    <col min="1" max="1" width="14.2857142857143" style="76" customWidth="1"/>
     <col min="2" max="2" width="47" customWidth="1"/>
     <col min="3" max="3" width="123.571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="65"/>
-      <c r="B2" s="65" t="s">
+      <c r="A2" s="71"/>
+      <c r="B2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="65"/>
-      <c r="B3" s="65" t="s">
+      <c r="A3" s="71"/>
+      <c r="B3" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="57" t="s">
+      <c r="C3" s="58" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="65"/>
-      <c r="B4" s="65" t="s">
+      <c r="A4" s="71"/>
+      <c r="B4" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="57" t="s">
+      <c r="C4" s="58" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="45" spans="1:3">
-      <c r="A5" s="65"/>
-      <c r="B5" s="65" t="s">
+      <c r="A5" s="71"/>
+      <c r="B5" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="69" t="s">
+      <c r="C5" s="75" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" s="65"/>
-      <c r="B6" s="69" t="s">
+      <c r="A6" s="71"/>
+      <c r="B6" s="75" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="57" t="s">
+      <c r="C6" s="58" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:3">
-      <c r="A7" s="65"/>
-      <c r="B7" s="65" t="s">
+      <c r="A7" s="71"/>
+      <c r="B7" s="71" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="13" t="s">
@@ -7018,8 +7148,8 @@
       </c>
     </row>
     <row r="8" spans="1:3">
-      <c r="A8" s="65"/>
-      <c r="B8" s="65" t="s">
+      <c r="A8" s="71"/>
+      <c r="B8" s="71" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="13" t="s">
@@ -7056,16 +7186,16 @@
         <v>16</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>18</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
     </row>
     <row r="2" s="2" customFormat="1" ht="17" customHeight="1" spans="1:6">
@@ -7084,7 +7214,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" s="2" customFormat="1" ht="180" spans="1:6">
@@ -7093,10 +7223,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" spans="1:6">
@@ -7116,7 +7246,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
@@ -7131,201 +7261,201 @@
         <v>56</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
     </row>
     <row r="8" s="2" customFormat="1" ht="74.25" spans="1:6">
       <c r="B8" s="6" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
     </row>
     <row r="9" s="2" customFormat="1" ht="409" customHeight="1" spans="1:6">
       <c r="B9" s="6" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="5" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" s="2" customFormat="1" ht="150" spans="1:6">
       <c r="B10" s="6" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
     </row>
     <row r="11" s="2" customFormat="1" ht="180" spans="1:6">
       <c r="B11" s="6" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C11" s="5"/>
       <c r="D11" s="2"/>
       <c r="E11" s="12" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
     </row>
     <row r="12" s="2" customFormat="1" ht="150" spans="1:6">
       <c r="B12" s="6" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C12" s="5"/>
       <c r="D12" s="2"/>
       <c r="E12" s="12" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
     </row>
     <row r="13" s="2" customFormat="1" ht="75" spans="1:6">
       <c r="B13" s="6" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
     </row>
     <row r="14" s="2" customFormat="1" ht="30" spans="1:6">
       <c r="B14" s="6" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" s="2" customFormat="1" ht="45" spans="1:6">
       <c r="B15" s="6" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
     </row>
     <row r="16" s="2" customFormat="1" ht="30" spans="1:6">
       <c r="B16" s="6" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
     </row>
     <row r="17" s="2" customFormat="1" ht="45" spans="2:6">
       <c r="B17" s="6" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
     </row>
     <row r="18" s="2" customFormat="1" ht="30" spans="2:6">
       <c r="B18" s="6" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="19" s="2" customFormat="1" ht="30" spans="2:6">
       <c r="B19" s="6" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
     </row>
     <row r="20" s="2" customFormat="1" ht="270" spans="2:6">
       <c r="B20" s="6" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="15" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" spans="2:6">
       <c r="B21" s="2" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="16" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
     </row>
     <row r="22" s="2" customFormat="1" ht="165" spans="2:6">
       <c r="B22" s="2" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" spans="2:6">
       <c r="B23" s="5" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
     </row>
     <row r="24" s="2" customFormat="1" ht="46" customHeight="1" spans="2:6">
       <c r="B24" s="5" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="D24" s="17"/>
     </row>
@@ -7346,24 +7476,24 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="14.7142857142857" style="65" customWidth="1"/>
-    <col min="2" max="2" width="28.2857142857143" style="65" customWidth="1"/>
-    <col min="3" max="3" width="62.7238095238095" style="65" customWidth="1"/>
-    <col min="4" max="4" width="54.5428571428571" style="65" customWidth="1"/>
+    <col min="1" max="1" width="14.7142857142857" style="71" customWidth="1"/>
+    <col min="2" max="2" width="28.2857142857143" style="71" customWidth="1"/>
+    <col min="3" max="3" width="62.7238095238095" style="71" customWidth="1"/>
+    <col min="4" max="4" width="54.5428571428571" style="71" customWidth="1"/>
     <col min="5" max="5" width="57" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="72" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="66" t="s">
+      <c r="B1" s="72" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="66" t="s">
+      <c r="C1" s="72" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="66" t="s">
+      <c r="D1" s="72" t="s">
         <v>18</v>
       </c>
       <c r="E1" s="3" t="s">
@@ -7371,32 +7501,32 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="73" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="67"/>
-      <c r="B3" s="65" t="s">
+      <c r="A3" s="73"/>
+      <c r="B3" s="71" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="65" t="s">
+      <c r="C3" s="71" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="67"/>
-      <c r="B4" s="65" t="s">
+      <c r="A4" s="73"/>
+      <c r="B4" s="71" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="68" t="s">
+      <c r="C4" s="74" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="65" t="s">
+      <c r="D4" s="71" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="5" s="64" customFormat="1" ht="61" customHeight="1" spans="1:5">
+    <row r="5" s="70" customFormat="1" ht="61" customHeight="1" spans="1:5">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>26</v>
@@ -7408,7 +7538,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" s="64" customFormat="1" ht="49" customHeight="1" spans="1:5">
+    <row r="6" s="70" customFormat="1" ht="49" customHeight="1" spans="1:5">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>29</v>
@@ -7418,7 +7548,7 @@
       </c>
       <c r="D6" s="5"/>
     </row>
-    <row r="7" s="64" customFormat="1" ht="316" customHeight="1" spans="1:5">
+    <row r="7" s="70" customFormat="1" ht="316" customHeight="1" spans="1:5">
       <c r="A7" s="2"/>
       <c r="B7" s="2" t="s">
         <v>31</v>
@@ -7429,27 +7559,27 @@
       <c r="D7" s="5"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="B8" s="65" t="s">
+      <c r="B8" s="71" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="65" t="s">
+      <c r="C8" s="71" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="69"/>
+      <c r="D8" s="75"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="65" t="s">
+      <c r="B9" s="71" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="65" t="s">
+      <c r="C9" s="71" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" ht="30" spans="1:5">
-      <c r="B10" s="65" t="s">
+      <c r="B10" s="71" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="69" t="s">
+      <c r="C10" s="75" t="s">
         <v>38</v>
       </c>
     </row>
@@ -7489,11 +7619,11 @@
       <c r="C17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E17" s="48" t="s">
+      <c r="E17" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="F17" s="48"/>
-      <c r="G17" s="48"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="49"/>
     </row>
     <row r="18" s="2" customFormat="1" ht="30" spans="1:7">
       <c r="B18" s="5" t="s">
@@ -7531,10 +7661,10 @@
       <c r="C22"/>
     </row>
     <row r="23" hidden="1" spans="1:7">
-      <c r="B23" s="65" t="s">
+      <c r="B23" s="71" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="69" t="s">
+      <c r="C23" s="75" t="s">
         <v>48</v>
       </c>
     </row>
@@ -7553,8 +7683,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E65"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
+  <dimension ref="A1:F69"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="13.1142857142857" customWidth="1"/>
     <col min="2" max="2" width="39.1428571428571" style="14" customWidth="1"/>
@@ -7601,7 +7731,7 @@
       <c r="B4" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="49" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="14" t="s">
@@ -7638,7 +7768,7 @@
       <c r="D7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="E7" s="48" t="s">
+      <c r="E7" s="49" t="s">
         <v>57</v>
       </c>
     </row>
@@ -7658,7 +7788,7 @@
       <c r="B9" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="59" t="s">
+      <c r="C9" s="61" t="s">
         <v>62</v>
       </c>
       <c r="E9" s="26"/>
@@ -7825,7 +7955,7 @@
       <c r="D24" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="E24" s="48" t="s">
+      <c r="E24" s="49" t="s">
         <v>102</v>
       </c>
     </row>
@@ -7854,7 +7984,7 @@
       <c r="C27" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="D27" s="60" t="s">
+      <c r="D27" s="62" t="s">
         <v>109</v>
       </c>
       <c r="E27" s="9" t="s">
@@ -7868,8 +7998,8 @@
       <c r="C28" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="D28" s="60"/>
-      <c r="E28" s="61"/>
+      <c r="D28" s="62"/>
+      <c r="E28" s="63"/>
     </row>
     <row r="29" ht="30" spans="2:5">
       <c r="B29" s="30" t="s">
@@ -7878,8 +8008,8 @@
       <c r="C29" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="D29" s="60"/>
-      <c r="E29" s="61"/>
+      <c r="D29" s="62"/>
+      <c r="E29" s="63"/>
     </row>
     <row r="30" ht="30" spans="2:5">
       <c r="B30" s="30" t="s">
@@ -7888,8 +8018,8 @@
       <c r="C30" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="D30" s="60"/>
-      <c r="E30" s="61"/>
+      <c r="D30" s="62"/>
+      <c r="E30" s="63"/>
     </row>
     <row r="31" spans="2:5">
       <c r="B31" s="30" t="s">
@@ -7898,7 +8028,7 @@
       <c r="C31" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="D31" s="60"/>
+      <c r="D31" s="62"/>
       <c r="E31" s="9"/>
     </row>
     <row r="32" ht="30" spans="2:5">
@@ -7908,7 +8038,7 @@
       <c r="C32" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D32" s="60" t="s">
+      <c r="D32" s="62" t="s">
         <v>119</v>
       </c>
       <c r="E32" s="9" t="s">
@@ -7922,8 +8052,8 @@
       <c r="C33" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="D33" s="60"/>
-      <c r="E33" s="61"/>
+      <c r="D33" s="62"/>
+      <c r="E33" s="63"/>
     </row>
     <row r="34" ht="30" spans="2:5">
       <c r="B34" s="30" t="s">
@@ -7932,8 +8062,8 @@
       <c r="C34" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="D34" s="60"/>
-      <c r="E34" s="61"/>
+      <c r="D34" s="62"/>
+      <c r="E34" s="63"/>
     </row>
     <row r="35" ht="30" spans="2:5">
       <c r="B35" s="30" t="s">
@@ -7942,8 +8072,8 @@
       <c r="C35" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="D35" s="60"/>
-      <c r="E35" s="61"/>
+      <c r="D35" s="62"/>
+      <c r="E35" s="63"/>
     </row>
     <row r="36" spans="2:5">
       <c r="B36" s="30" t="s">
@@ -7952,8 +8082,8 @@
       <c r="C36" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D36" s="60"/>
-      <c r="E36" s="61"/>
+      <c r="D36" s="62"/>
+      <c r="E36" s="63"/>
     </row>
     <row r="37" spans="2:5">
       <c r="B37" s="30" t="s">
@@ -7962,10 +8092,10 @@
       <c r="C37" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="D37" s="60" t="s">
+      <c r="D37" s="62" t="s">
         <v>125</v>
       </c>
-      <c r="E37" s="61"/>
+      <c r="E37" s="63"/>
     </row>
     <row r="38" ht="45" spans="2:5">
       <c r="B38" s="30" t="s">
@@ -7974,32 +8104,32 @@
       <c r="C38" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="D38" s="60"/>
-      <c r="E38" s="71" t="s">
+      <c r="D38" s="62"/>
+      <c r="E38" s="77" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="39" ht="135" spans="2:5">
-      <c r="B39" s="62" t="s">
+      <c r="B39" s="64" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="62"/>
-      <c r="D39" s="62" t="s">
+      <c r="C39" s="64"/>
+      <c r="D39" s="64" t="s">
         <v>130</v>
       </c>
-      <c r="E39" s="26" t="s">
+      <c r="E39" s="65" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="40" ht="135" spans="2:5">
-      <c r="B40" s="62" t="s">
+      <c r="B40" s="64" t="s">
         <v>132</v>
       </c>
-      <c r="C40" s="62"/>
-      <c r="D40" s="62" t="s">
+      <c r="C40" s="64"/>
+      <c r="D40" s="64" t="s">
         <v>133</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E40" s="65" t="s">
         <v>131</v>
       </c>
     </row>
@@ -8058,10 +8188,10 @@
       <c r="C46" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="D46" s="57" t="s">
+      <c r="D46" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="E46" s="48" t="s">
+      <c r="E46" s="49" t="s">
         <v>147</v>
       </c>
     </row>
@@ -8086,7 +8216,7 @@
       </c>
       <c r="E48" s="26"/>
     </row>
-    <row r="49" spans="2:5">
+    <row r="49" spans="2:6">
       <c r="B49" s="14" t="s">
         <v>152</v>
       </c>
@@ -8095,7 +8225,7 @@
       </c>
       <c r="E49" s="26"/>
     </row>
-    <row r="50" spans="2:5">
+    <row r="50" spans="2:6">
       <c r="B50" s="14" t="s">
         <v>154</v>
       </c>
@@ -8104,7 +8234,7 @@
       </c>
       <c r="E50" s="26"/>
     </row>
-    <row r="51" spans="2:5">
+    <row r="51" spans="2:6">
       <c r="B51" s="14" t="s">
         <v>156</v>
       </c>
@@ -8113,7 +8243,7 @@
       </c>
       <c r="E51" s="26"/>
     </row>
-    <row r="52" ht="150" spans="2:5">
+    <row r="52" ht="150" spans="2:6">
       <c r="B52" s="14" t="s">
         <v>157</v>
       </c>
@@ -8127,7 +8257,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="53" spans="2:5">
+    <row r="53" spans="2:6">
       <c r="B53" s="14" t="s">
         <v>161</v>
       </c>
@@ -8136,7 +8266,7 @@
       </c>
       <c r="E53" s="26"/>
     </row>
-    <row r="54" spans="2:5">
+    <row r="54" spans="2:6">
       <c r="B54" s="14" t="s">
         <v>163</v>
       </c>
@@ -8145,7 +8275,7 @@
       </c>
       <c r="E54" s="26"/>
     </row>
-    <row r="55" spans="2:5">
+    <row r="55" spans="2:6">
       <c r="B55" s="14" t="s">
         <v>164</v>
       </c>
@@ -8154,7 +8284,7 @@
       </c>
       <c r="E55" s="26"/>
     </row>
-    <row r="56" spans="2:5">
+    <row r="56" spans="2:6">
       <c r="B56" s="14" t="s">
         <v>166</v>
       </c>
@@ -8163,7 +8293,7 @@
       </c>
       <c r="E56" s="26"/>
     </row>
-    <row r="57" spans="2:5">
+    <row r="57" spans="2:6">
       <c r="B57" s="14" t="s">
         <v>168</v>
       </c>
@@ -8172,7 +8302,7 @@
       </c>
       <c r="E57" s="26"/>
     </row>
-    <row r="58" spans="2:5">
+    <row r="58" spans="2:6">
       <c r="B58" s="14" t="s">
         <v>169</v>
       </c>
@@ -8181,7 +8311,7 @@
       </c>
       <c r="E58" s="26"/>
     </row>
-    <row r="59" ht="180" spans="2:5">
+    <row r="59" ht="180" spans="2:6">
       <c r="B59" s="14" t="s">
         <v>171</v>
       </c>
@@ -8193,7 +8323,7 @@
       </c>
       <c r="E59" s="26"/>
     </row>
-    <row r="60" ht="255" spans="2:5">
+    <row r="60" ht="255" spans="2:6">
       <c r="B60" s="14" t="s">
         <v>174</v>
       </c>
@@ -8207,30 +8337,74 @@
         <v>177</v>
       </c>
     </row>
-    <row r="61" spans="2:5">
-      <c r="B61" s="14" t="s">
+    <row r="61" s="60" customFormat="1" ht="45" spans="2:6">
+      <c r="B61" s="66" t="s">
         <v>178</v>
       </c>
-      <c r="C61" s="14" t="s">
+      <c r="C61" s="66" t="s">
         <v>179</v>
       </c>
-      <c r="D61" s="63" t="s">
+      <c r="D61" s="67"/>
+      <c r="E61" s="66"/>
+      <c r="F61" s="66"/>
+    </row>
+    <row r="62" s="60" customFormat="1" spans="2:6">
+      <c r="B62" s="66" t="s">
         <v>180</v>
       </c>
-      <c r="E61" s="26"/>
-    </row>
-    <row r="62" ht="42.95" customHeight="1" spans="2:5">
-      <c r="B62" s="14" t="s">
+      <c r="C62" s="66" t="s">
         <v>181</v>
       </c>
-      <c r="C62" s="59" t="s">
+      <c r="D62" s="67"/>
+      <c r="E62" s="66"/>
+      <c r="F62" s="66"/>
+    </row>
+    <row r="63" s="60" customFormat="1" ht="195" spans="2:6">
+      <c r="B63" s="66" t="s">
         <v>182</v>
       </c>
-      <c r="D62" s="63"/>
-      <c r="E62" s="26"/>
-    </row>
-    <row r="65" spans="3:3">
-      <c r="C65" s="59"/>
+      <c r="C63" s="66"/>
+      <c r="D63" s="67"/>
+      <c r="E63" s="68" t="s">
+        <v>183</v>
+      </c>
+      <c r="F63" s="66"/>
+    </row>
+    <row r="64" s="60" customFormat="1" spans="2:6">
+      <c r="B64" s="66" t="s">
+        <v>184</v>
+      </c>
+      <c r="C64" s="67" t="s">
+        <v>185</v>
+      </c>
+      <c r="D64" s="67"/>
+      <c r="E64" s="68"/>
+      <c r="F64" s="66"/>
+    </row>
+    <row r="65" spans="2:5">
+      <c r="B65" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="D65" s="69" t="s">
+        <v>188</v>
+      </c>
+      <c r="E65" s="26"/>
+    </row>
+    <row r="66" ht="42.95" customHeight="1" spans="2:5">
+      <c r="B66" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="C66" s="61" t="s">
+        <v>190</v>
+      </c>
+      <c r="D66" s="69"/>
+      <c r="E66" s="26"/>
+    </row>
+    <row r="69" spans="2:5">
+      <c r="C69" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -8238,11 +8412,11 @@
     <mergeCell ref="D27:D31"/>
     <mergeCell ref="D32:D36"/>
     <mergeCell ref="D37:D38"/>
-    <mergeCell ref="D61:D62"/>
+    <mergeCell ref="D65:D66"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C9" r:id="rId1" display="&quot;http://shinny.org/us/ny/hrsn/StructureDefinition/middle-name&quot;" tooltip="http://shinny.org/us/ny/hrsn/StructureDefinition/middle-name"/>
-    <hyperlink ref="C62" r:id="rId2" display="&quot;http://shinny.org/us/ny/hrsn/Patient/&lt;id&gt;&quot;" tooltip="http://shinny.org/us/ny/hrsn/Patient/PID.3.1"/>
+    <hyperlink ref="C66" r:id="rId2" display="&quot;http://shinny.org/us/ny/hrsn/Patient/&lt;id&gt;&quot;" tooltip="http://shinny.org/us/ny/hrsn/Patient/PID.3.1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1.39370078740157" bottom="1.39370078740157" header="1" footer="1"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
@@ -8285,19 +8459,19 @@
       <c r="A2" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="53" t="s">
-        <v>183</v>
-      </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
+      <c r="B2" s="54" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
     </row>
     <row r="3" spans="1:5">
       <c r="B3" s="14" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="E3" s="26"/>
     </row>
@@ -8305,11 +8479,11 @@
       <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="54" t="s">
-        <v>185</v>
+      <c r="C4" s="55" t="s">
+        <v>193</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E4" s="26"/>
     </row>
@@ -8318,7 +8492,7 @@
         <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="E5" s="26"/>
     </row>
@@ -8327,206 +8501,206 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E6" s="26"/>
     </row>
     <row r="7" ht="45" spans="1:5">
       <c r="B7" s="21" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C7" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="D7" t="s">
-        <v>191</v>
-      </c>
-      <c r="E7" s="54" t="s">
-        <v>192</v>
+        <v>199</v>
+      </c>
+      <c r="E7" s="55" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="8" ht="135" spans="1:5">
-      <c r="B8" s="55" t="s">
-        <v>193</v>
+      <c r="B8" s="56" t="s">
+        <v>201</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>194</v>
-      </c>
-      <c r="D8" s="56" t="s">
-        <v>195</v>
+        <v>202</v>
+      </c>
+      <c r="D8" s="57" t="s">
+        <v>203</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="55" t="s">
-        <v>197</v>
+      <c r="B9" s="56" t="s">
+        <v>205</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="D9" s="29"/>
       <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="B10" s="55" t="s">
-        <v>199</v>
+      <c r="B10" s="56" t="s">
+        <v>207</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="D10" s="29"/>
       <c r="E10" s="26" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
     </row>
     <row r="11" ht="225" spans="1:5">
       <c r="B11" s="21" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="D11" s="57" t="s">
-        <v>204</v>
+        <v>211</v>
+      </c>
+      <c r="D11" s="58" t="s">
+        <v>212</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="B12" s="21" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="B13" s="21" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" ht="30" spans="1:5">
       <c r="B14" s="21" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C14" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="D14" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="15" ht="135" spans="1:5">
       <c r="B15" s="21" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="C15" s="30" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="D15" s="30" t="s">
-        <v>215</v>
-      </c>
-      <c r="E15" s="54" t="s">
-        <v>216</v>
+        <v>223</v>
+      </c>
+      <c r="E15" s="55" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="16" ht="45" spans="1:5">
       <c r="B16" s="21" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="E16" s="26"/>
     </row>
     <row r="17" ht="60" spans="2:5">
-      <c r="B17" s="55" t="s">
-        <v>220</v>
-      </c>
-      <c r="C17" s="58" t="s">
-        <v>221</v>
+      <c r="B17" s="56" t="s">
+        <v>228</v>
+      </c>
+      <c r="C17" s="59" t="s">
+        <v>229</v>
       </c>
       <c r="D17" s="30" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="E17" s="26"/>
     </row>
     <row r="18" ht="60" spans="2:5">
-      <c r="B18" s="58" t="s">
-        <v>223</v>
-      </c>
-      <c r="C18" s="58" t="s">
-        <v>224</v>
+      <c r="B18" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="C18" s="59" t="s">
+        <v>232</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="6" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="D19" s="30" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" s="6" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="D20" s="30"/>
       <c r="E20" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="21" ht="77" customHeight="1" spans="2:5">
       <c r="B21" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="E21" s="26"/>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="26"/>
@@ -8584,7 +8758,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="E3" s="26"/>
     </row>
@@ -8593,11 +8767,11 @@
       <c r="B4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="48" t="s">
-        <v>234</v>
+      <c r="C4" s="49" t="s">
+        <v>242</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="E4" s="26"/>
     </row>
@@ -8617,265 +8791,265 @@
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="26"/>
     </row>
     <row r="7" spans="1:5">
       <c r="B7" s="21" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" ht="75" spans="1:5">
       <c r="B8" s="21" t="s">
-        <v>238</v>
-      </c>
-      <c r="C8" s="52" t="s">
-        <v>239</v>
+        <v>246</v>
+      </c>
+      <c r="C8" s="53" t="s">
+        <v>247</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="E8" s="72" t="s">
-        <v>241</v>
+        <v>248</v>
+      </c>
+      <c r="E8" s="78" t="s">
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="B9" s="21" t="s">
-        <v>242</v>
-      </c>
-      <c r="C9" s="52" t="s">
-        <v>243</v>
+        <v>250</v>
+      </c>
+      <c r="C9" s="53" t="s">
+        <v>251</v>
       </c>
       <c r="D9" s="14"/>
       <c r="E9" s="26"/>
     </row>
     <row r="10" ht="75" spans="1:5">
       <c r="B10" s="21" t="s">
-        <v>244</v>
-      </c>
-      <c r="C10" s="52" t="s">
-        <v>245</v>
+        <v>252</v>
+      </c>
+      <c r="C10" s="53" t="s">
+        <v>253</v>
       </c>
       <c r="D10" s="14"/>
-      <c r="E10" s="72" t="s">
-        <v>246</v>
+      <c r="E10" s="78" t="s">
+        <v>254</v>
       </c>
     </row>
     <row r="11" ht="120" spans="1:5">
       <c r="B11" s="21" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="E11" s="48" t="s">
-        <v>250</v>
+        <v>257</v>
+      </c>
+      <c r="E11" s="49" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="12" ht="60" spans="1:5">
       <c r="B12" s="21" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="B13" s="21" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="E13" s="26"/>
     </row>
     <row r="14" spans="1:5">
       <c r="B14" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="C14" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="E14" s="26"/>
     </row>
     <row r="15" ht="75" spans="1:5">
       <c r="B15" s="21" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C15" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="E15" s="26"/>
     </row>
     <row r="16" ht="30" spans="1:5">
       <c r="B16" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="E16" s="26"/>
     </row>
     <row r="17" ht="60" spans="2:5">
       <c r="B17" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="E17" s="26"/>
     </row>
     <row r="18" spans="2:5">
       <c r="B18" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="E18" s="26"/>
     </row>
     <row r="19" ht="30" spans="2:5">
       <c r="B19" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="E19" s="26" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
     </row>
     <row r="20" spans="2:5">
       <c r="B20" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="D20" s="14"/>
       <c r="E20" s="26" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="21" spans="2:5">
       <c r="B21" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="26" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" spans="2:5">
       <c r="B22" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="26" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="23" ht="30" spans="2:5">
       <c r="B23" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="D23" s="14"/>
       <c r="E23" s="26" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" ht="75" spans="2:5">
       <c r="B24" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C24" s="14"/>
       <c r="D24" s="14" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="E24" s="26"/>
     </row>
     <row r="25" spans="2:5">
       <c r="B25" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="D25" s="14"/>
       <c r="E25" s="26"/>
     </row>
     <row r="26" ht="60" spans="2:5">
       <c r="B26" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="E26" s="26" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
     </row>
     <row r="27" spans="2:5">
       <c r="B27" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="D27" s="14"/>
       <c r="E27" s="26" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" customHeight="1" spans="2:5">
       <c r="B28" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="E28" s="26"/>
     </row>
     <row r="29" ht="30" spans="2:5">
       <c r="B29" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="D29" s="14"/>
       <c r="E29" s="26"/>
@@ -8923,7 +9097,7 @@
         <v>19</v>
       </c>
       <c r="F1" s="35" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8937,7 +9111,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E3" s="36"/>
     </row>
@@ -8946,10 +9120,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="E4" s="36"/>
     </row>
@@ -8969,61 +9143,61 @@
         <v>29</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="D6" s="37"/>
       <c r="E6" s="36"/>
     </row>
     <row r="7" ht="30" spans="1:6">
       <c r="B7" s="38" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="C7" s="39"/>
       <c r="D7" s="39" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="F7" s="40"/>
     </row>
     <row r="8" ht="195" spans="1:6">
       <c r="B8" s="33" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C8" s="41" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9" s="33" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="D9" s="37"/>
       <c r="E9" s="36"/>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" s="37" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="D10" s="37"/>
       <c r="E10" s="36"/>
     </row>
     <row r="11" ht="30" spans="1:6">
       <c r="B11" s="37" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>135</v>
@@ -9033,51 +9207,51 @@
     </row>
     <row r="12" ht="30" spans="1:6">
       <c r="B12" s="37" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="D12" s="37"/>
       <c r="E12" s="36"/>
     </row>
     <row r="13" ht="225" spans="1:6">
       <c r="B13" s="33" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="E13" s="42" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="B14" s="33" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D14" s="37"/>
       <c r="E14" s="36"/>
     </row>
     <row r="15" spans="1:6">
       <c r="B15" s="37" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="D15" s="37"/>
       <c r="E15" s="36"/>
     </row>
     <row r="16" ht="30" spans="1:6">
       <c r="B16" s="37" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>135</v>
@@ -9087,49 +9261,49 @@
     </row>
     <row r="17" ht="30" spans="2:6">
       <c r="B17" s="37" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="D17" s="37"/>
       <c r="E17" s="36"/>
     </row>
     <row r="18" ht="30" spans="2:6">
       <c r="B18" s="43" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="C18" s="44" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="E18" s="42" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="19" ht="135" spans="2:6">
       <c r="B19" s="39" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C19" s="45"/>
       <c r="D19" s="46" t="s">
-        <v>326</v>
-      </c>
-      <c r="E19" s="36" t="s">
-        <v>327</v>
+        <v>334</v>
+      </c>
+      <c r="E19" s="47" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="20" ht="75" spans="2:6">
       <c r="B20" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="47" t="s">
-        <v>328</v>
+      <c r="C20" s="48" t="s">
+        <v>336</v>
       </c>
       <c r="D20" s="37"/>
-      <c r="E20" s="48" t="s">
+      <c r="E20" s="49" t="s">
         <v>102</v>
       </c>
     </row>
@@ -9137,11 +9311,11 @@
       <c r="B21" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="C21" s="47" t="s">
-        <v>329</v>
+      <c r="C21" s="48" t="s">
+        <v>337</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="E21" s="36"/>
     </row>
@@ -9149,22 +9323,22 @@
       <c r="B22" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="C22" s="49" t="s">
-        <v>331</v>
+      <c r="C22" s="50" t="s">
+        <v>339</v>
       </c>
       <c r="D22" s="37"/>
       <c r="E22" s="15"/>
-      <c r="F22" s="50"/>
+      <c r="F22" s="51"/>
     </row>
     <row r="23" spans="2:6">
       <c r="B23" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="51" t="s">
-        <v>332</v>
+      <c r="C23" s="52" t="s">
+        <v>340</v>
       </c>
       <c r="D23" s="37" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="E23" s="36"/>
     </row>
@@ -9172,20 +9346,20 @@
       <c r="B24" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="C24" s="47" t="s">
-        <v>334</v>
+      <c r="C24" s="48" t="s">
+        <v>342</v>
       </c>
       <c r="D24" s="37"/>
       <c r="E24" s="31" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
     </row>
     <row r="25" ht="30" spans="2:6">
       <c r="B25" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="51" t="s">
-        <v>336</v>
+      <c r="C25" s="52" t="s">
+        <v>344</v>
       </c>
       <c r="D25" s="37"/>
       <c r="E25" s="36"/>
@@ -9194,8 +9368,8 @@
       <c r="B26" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="C26" s="47" t="s">
-        <v>337</v>
+      <c r="C26" s="48" t="s">
+        <v>345</v>
       </c>
       <c r="D26" s="37"/>
       <c r="E26" s="36"/>
@@ -9204,8 +9378,8 @@
       <c r="B27" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C27" s="47" t="s">
-        <v>338</v>
+      <c r="C27" s="48" t="s">
+        <v>346</v>
       </c>
       <c r="D27" s="37"/>
       <c r="E27" s="36"/>
@@ -9214,8 +9388,8 @@
       <c r="B28" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="C28" s="47" t="s">
-        <v>339</v>
+      <c r="C28" s="48" t="s">
+        <v>347</v>
       </c>
       <c r="D28" s="37"/>
       <c r="E28" s="36"/>
@@ -9224,30 +9398,30 @@
       <c r="B29" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="C29" s="47" t="s">
-        <v>340</v>
+      <c r="C29" s="48" t="s">
+        <v>348</v>
       </c>
       <c r="D29" s="37"/>
       <c r="E29" s="36"/>
     </row>
     <row r="30" customHeight="1" spans="2:6">
       <c r="B30" s="37" t="s">
-        <v>178</v>
-      </c>
-      <c r="C30" s="47" t="s">
-        <v>179</v>
+        <v>186</v>
+      </c>
+      <c r="C30" s="48" t="s">
+        <v>187</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="E30" s="36"/>
     </row>
     <row r="31" ht="30" spans="2:6">
       <c r="B31" s="37" t="s">
-        <v>181</v>
-      </c>
-      <c r="C31" s="51" t="s">
-        <v>342</v>
+        <v>189</v>
+      </c>
+      <c r="C31" s="52" t="s">
+        <v>350</v>
       </c>
       <c r="D31" s="37"/>
       <c r="E31" s="36"/>
@@ -9304,7 +9478,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E3" s="14"/>
     </row>
@@ -9313,10 +9487,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E4" s="14"/>
     </row>
@@ -9334,7 +9508,7 @@
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="E6" s="14"/>
     </row>
@@ -9347,310 +9521,310 @@
         <v>56</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="8" ht="74.25" spans="1:5">
       <c r="B8" s="22" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9" ht="120" spans="1:5">
       <c r="B9" s="28" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C9" s="29"/>
       <c r="D9" s="30" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" ht="45" spans="1:5">
       <c r="A10" s="29"/>
       <c r="B10" s="6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D10" s="30"/>
       <c r="E10" s="9" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" ht="210" spans="1:5">
       <c r="A11" s="29"/>
       <c r="B11" s="6" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="30"/>
       <c r="E11" s="12" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
     </row>
     <row r="12" ht="210" spans="1:5">
       <c r="A12" s="29"/>
       <c r="B12" s="6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="30"/>
       <c r="E12" s="12" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="29"/>
       <c r="B13" s="6" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="30"/>
       <c r="E13" s="9" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
     </row>
     <row r="14" ht="150" spans="1:5">
       <c r="B14" s="14" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5">
       <c r="B15" s="22" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" s="22" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="E16" s="14"/>
     </row>
     <row r="17" spans="2:5">
       <c r="B17" s="14" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="E17" s="14"/>
     </row>
     <row r="18" ht="105" spans="2:5">
       <c r="B18" s="14" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="19" ht="30" spans="2:5">
       <c r="B19" s="14" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="20" ht="30" spans="2:5">
       <c r="B20" s="14" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="21" s="2" customFormat="1" ht="37" customHeight="1" spans="2:5">
       <c r="B21" s="8" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="E21" s="9"/>
     </row>
     <row r="22" s="2" customFormat="1" ht="45" spans="2:5">
       <c r="B22" s="8" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D22" s="17"/>
       <c r="E22" s="31" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="23" s="2" customFormat="1" ht="45" spans="2:5">
       <c r="B23" s="8" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="17"/>
       <c r="E23" s="12" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="24" ht="75" spans="2:5">
       <c r="B24" s="22" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="E24" s="14"/>
     </row>
     <row r="25" ht="30" spans="2:5">
       <c r="B25" s="22" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="E25" s="14"/>
     </row>
     <row r="26" ht="45" spans="2:5">
       <c r="B26" s="28" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="D26" s="30" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="E26" s="14"/>
     </row>
     <row r="27" ht="30" spans="2:5">
       <c r="B27" s="22" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
     <row r="28" ht="60" spans="2:5">
       <c r="B28" s="14" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="E28" s="14"/>
     </row>
     <row r="29" s="2" customFormat="1" ht="30" spans="2:5">
       <c r="B29" s="6" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
     </row>
     <row r="30" s="2" customFormat="1" spans="2:5">
       <c r="B30" s="6" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
     </row>
     <row r="31" s="2" customFormat="1" ht="270" spans="2:5">
       <c r="B31" s="6" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="C31" s="5"/>
       <c r="D31" s="5"/>
       <c r="E31" s="15" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
     </row>
     <row r="32" ht="30" spans="2:5">
       <c r="B32" s="14" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="E32" s="14"/>
     </row>
     <row r="33" spans="2:5">
       <c r="B33" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="E33" s="14"/>
     </row>
     <row r="34" ht="78" customHeight="1" spans="2:5">
       <c r="B34" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C34" s="32" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
@@ -9707,7 +9881,7 @@
     </row>
     <row r="2" ht="30" spans="1:5">
       <c r="A2" s="25" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="E2" s="26"/>
     </row>
@@ -9717,7 +9891,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="E3" s="26"/>
     </row>
@@ -9727,10 +9901,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="E4" s="26"/>
     </row>
@@ -9750,152 +9924,152 @@
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="26"/>
     </row>
     <row r="7" ht="74.25" spans="1:5">
       <c r="B7" s="21" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C7" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="D7" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="B8" s="21" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C8" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D8" s="14"/>
       <c r="E8" s="26"/>
     </row>
     <row r="9" ht="42.95" customHeight="1" spans="1:5">
       <c r="B9" s="21" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C9" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="E9" s="26"/>
     </row>
     <row r="10" spans="1:5">
       <c r="B10" s="21" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="D10" s="14"/>
       <c r="E10" s="26"/>
     </row>
     <row r="11" ht="60.95" customHeight="1" spans="1:5">
       <c r="B11" s="21" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="D11" s="14"/>
       <c r="E11" s="26"/>
     </row>
     <row r="12" ht="30" spans="1:5">
       <c r="B12" s="14" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="E12" s="26"/>
     </row>
     <row r="13" ht="30" spans="1:5">
       <c r="B13" s="14" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="D13" s="14"/>
       <c r="E13" s="26"/>
     </row>
     <row r="14" ht="78" customHeight="1" spans="1:5">
       <c r="B14" s="14" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="D14" s="14"/>
       <c r="E14" s="26"/>
     </row>
     <row r="15" ht="45" spans="1:5">
       <c r="B15" s="21" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="E15" s="26"/>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="E16" s="26"/>
     </row>
     <row r="17" ht="30" spans="2:5">
       <c r="B17" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C17" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="D17" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="E17" s="26" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
     </row>
     <row r="18" customHeight="1" spans="2:5">
       <c r="B18" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="E18" s="26"/>
     </row>
     <row r="19" spans="2:5">
       <c r="B19" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="D19" s="14"/>
       <c r="E19" s="26"/>
@@ -9952,7 +10126,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -9961,10 +10135,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="D4" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -9983,125 +10157,125 @@
         <v>29</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="D6" s="14"/>
       <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5">
       <c r="B7" s="21" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="D7" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="E7" s="23"/>
     </row>
     <row r="8" ht="165" spans="1:5">
       <c r="B8" s="21" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="E8" s="24"/>
     </row>
     <row r="9" spans="1:5">
       <c r="B9" s="21" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="B10" s="21" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="B11" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
     </row>
     <row r="12" ht="90" spans="1:5">
       <c r="B12" s="21" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
     </row>
     <row r="13" ht="45" spans="1:5">
       <c r="B13" s="21" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" ht="75" spans="1:5">
       <c r="B14" s="21" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
     </row>
     <row r="15" ht="90" spans="1:5">
       <c r="B15" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="B16" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
     </row>
     <row r="17" customHeight="1" spans="2:4">
       <c r="B17" s="14" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
     </row>
     <row r="18" ht="30" spans="2:4">
       <c r="B18" s="14" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="D18" s="14"/>
     </row>

</xml_diff>